<commit_message>
🔄 Update Excel template for LCA dashboard
</commit_message>
<xml_diff>
--- a/assets/template_LCA.xlsx
+++ b/assets/template_LCA.xlsx
@@ -5,18 +5,21 @@
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\idriouech001\Desktop\BIOCOP Project\Code contribution analysis\Full version\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\idriouech001\Desktop\BIOCOP Project\Code contribution analysis\Final\assets\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7952DC6F-20A8-4F5A-BFE4-0DBCC8B497D9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{81FCDBEC-1B92-47E3-9042-CF28FA45A620}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-19320" yWindow="-1755" windowWidth="19440" windowHeight="14880" xr2:uid="{CEBC2EDF-78AC-4BE7-A36B-72086DC8A7D5}"/>
+    <workbookView xWindow="-19320" yWindow="-1755" windowWidth="19440" windowHeight="14880" activeTab="4" xr2:uid="{CEBC2EDF-78AC-4BE7-A36B-72086DC8A7D5}"/>
   </bookViews>
   <sheets>
     <sheet name="User guide" sheetId="8" r:id="rId1"/>
     <sheet name="Template" sheetId="1" r:id="rId2"/>
+    <sheet name="Exemple 1" sheetId="9" r:id="rId3"/>
+    <sheet name="Exemple 2" sheetId="10" r:id="rId4"/>
+    <sheet name="Exemple 3" sheetId="11" r:id="rId5"/>
   </sheets>
-  <calcPr calcId="191029"/>
+  <calcPr calcId="191029" iterate="1" iterateCount="200" iterateDelta="9.9999999999999995E-8" calcOnSave="0"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
@@ -35,7 +38,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="141" uniqueCount="19">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="270" uniqueCount="87">
   <si>
     <t>Catégorie d'impact</t>
   </si>
@@ -391,12 +394,263 @@
 One integrated bar chart that shows stacked contributions for all scenarios and categories, with optional hatching for clarity.</t>
     </r>
   </si>
+  <si>
+    <t>SC1 (sc1. Lab, 400°C)</t>
+  </si>
+  <si>
+    <t>SC2 (sc2. Industrial, calcium nitrate, 325°C)</t>
+  </si>
+  <si>
+    <t>SC3 (sc3. Industrial, calcium nitrate, 400°C)</t>
+  </si>
+  <si>
+    <t>SC4 (sc4. Industrial, calcium chloride, 400°C)</t>
+  </si>
+  <si>
+    <t>Si-source</t>
+  </si>
+  <si>
+    <t>Ca-source (Calcium nitrate)</t>
+  </si>
+  <si>
+    <t>Water</t>
+  </si>
+  <si>
+    <t>Heat</t>
+  </si>
+  <si>
+    <t>Wastewater</t>
+  </si>
+  <si>
+    <t>Ca-source (Calcium chloride)</t>
+  </si>
+  <si>
+    <t>GW (kg CO₂ eq)</t>
+  </si>
+  <si>
+    <t>MEut (kg N eq)</t>
+  </si>
+  <si>
+    <t>FEut (kg P eq)</t>
+  </si>
+  <si>
+    <t>SOD (kg CFC11 eq)</t>
+  </si>
+  <si>
+    <t>OF (kg NMVOC)</t>
+  </si>
+  <si>
+    <t>IR (kBq Co-60 eq)</t>
+  </si>
+  <si>
+    <t>HCT (CTUh)</t>
+  </si>
+  <si>
+    <t>HNCT (CTUh)</t>
+  </si>
+  <si>
+    <t>FWEco (kg 1,4-DCB eq)</t>
+  </si>
+  <si>
+    <t>MEco (kg 1,4-DCB eq)</t>
+  </si>
+  <si>
+    <t>TEco (kg 1,4-DCB eq)</t>
+  </si>
+  <si>
+    <t>TA (kg SO₂ eq)</t>
+  </si>
+  <si>
+    <t>FPMF (kg PM2.5 eq)</t>
+  </si>
+  <si>
+    <t>FRS (kg oil eq)</t>
+  </si>
+  <si>
+    <t>MRS (kg Cu eq)</t>
+  </si>
+  <si>
+    <t>LU (m²a crop eq)</t>
+  </si>
+  <si>
+    <t>WC (m³)</t>
+  </si>
+  <si>
+    <t>CED (MJ)</t>
+  </si>
+  <si>
+    <t>Scénario 1 (lab)</t>
+  </si>
+  <si>
+    <t>Scénario 2  (upscale)</t>
+  </si>
+  <si>
+    <t>Scénario 3 (hybrid)</t>
+  </si>
+  <si>
+    <t>TEP</t>
+  </si>
+  <si>
+    <t>co2</t>
+  </si>
+  <si>
+    <t>electricité</t>
+  </si>
+  <si>
+    <t>fin de vie</t>
+  </si>
+  <si>
+    <t>production</t>
+  </si>
+  <si>
+    <t>extraction</t>
+  </si>
+  <si>
+    <t>chromato</t>
+  </si>
+  <si>
+    <t>equipement</t>
+  </si>
+  <si>
+    <t>transport</t>
+  </si>
+  <si>
+    <t>réacteur</t>
+  </si>
+  <si>
+    <t>cc</t>
+  </si>
+  <si>
+    <t>ta</t>
+  </si>
+  <si>
+    <t>cht</t>
+  </si>
+  <si>
+    <t>sod</t>
+  </si>
+  <si>
+    <t>fpmf</t>
+  </si>
+  <si>
+    <t>wc</t>
+  </si>
+  <si>
+    <t>frs</t>
+  </si>
+  <si>
+    <t>mrs</t>
+  </si>
+  <si>
+    <r>
+      <t>Scénario 1 (</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FFFF0000"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>Lab, 400°C</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>)</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t>Scénario 2 (</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FFFF0000"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>Industrial, calcium nitrate, 325°C</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>)</t>
+    </r>
+  </si>
+  <si>
+    <t>CC</t>
+  </si>
+  <si>
+    <t>SOD</t>
+  </si>
+  <si>
+    <t>OF, HH</t>
+  </si>
+  <si>
+    <t>OF, TE</t>
+  </si>
+  <si>
+    <t>IR</t>
+  </si>
+  <si>
+    <t>HCT</t>
+  </si>
+  <si>
+    <t>HN-CT</t>
+  </si>
+  <si>
+    <t>FE</t>
+  </si>
+  <si>
+    <t>ME</t>
+  </si>
+  <si>
+    <t>TE</t>
+  </si>
+  <si>
+    <t>TA</t>
+  </si>
+  <si>
+    <t>FPMF</t>
+  </si>
+  <si>
+    <t>FRS</t>
+  </si>
+  <si>
+    <t>MRS</t>
+  </si>
+  <si>
+    <t>LU</t>
+  </si>
+  <si>
+    <t>WC</t>
+  </si>
+  <si>
+    <t>CED</t>
+  </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="13" x14ac:knownFonts="1">
+  <numFmts count="1">
+    <numFmt numFmtId="168" formatCode="0.0000000000"/>
+  </numFmts>
+  <fonts count="19" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -489,8 +743,45 @@
       <name val="Arial"/>
       <family val="2"/>
     </font>
+    <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color indexed="2"/>
+      <name val="Calibri"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FF000000"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
   </fonts>
-  <fills count="8">
+  <fills count="18">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -533,8 +824,68 @@
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="2" tint="-9.9978637043366805E-2"/>
+        <bgColor theme="2" tint="-9.9978637043366805E-2"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="4" tint="0.79998168889431442"/>
+        <bgColor theme="4" tint="0.79998168889431442"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="5" tint="0.79998168889431442"/>
+        <bgColor theme="5" tint="0.79998168889431442"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="9" tint="0.59999389629810485"/>
+        <bgColor theme="9" tint="0.59999389629810485"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="0" tint="-4.9989318521683403E-2"/>
+        <bgColor theme="0" tint="-4.9989318521683403E-2"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="4" tint="0.59999389629810485"/>
+        <bgColor theme="4" tint="0.59999389629810485"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="7" tint="0.59999389629810485"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFD9E2F3"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFF2F2F2"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFE597"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="12">
+  <borders count="22">
     <border>
       <left/>
       <right/>
@@ -691,11 +1042,152 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color auto="1"/>
+      </left>
+      <right style="thin">
+        <color auto="1"/>
+      </right>
+      <top style="thin">
+        <color auto="1"/>
+      </top>
+      <bottom style="thin">
+        <color auto="1"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color auto="1"/>
+      </left>
+      <right style="medium">
+        <color auto="1"/>
+      </right>
+      <top style="medium">
+        <color auto="1"/>
+      </top>
+      <bottom style="thin">
+        <color auto="1"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color auto="1"/>
+      </left>
+      <right style="medium">
+        <color auto="1"/>
+      </right>
+      <top style="thin">
+        <color auto="1"/>
+      </top>
+      <bottom style="thin">
+        <color auto="1"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color auto="1"/>
+      </left>
+      <right style="medium">
+        <color auto="1"/>
+      </right>
+      <top style="thin">
+        <color auto="1"/>
+      </top>
+      <bottom style="medium">
+        <color auto="1"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color auto="1"/>
+      </left>
+      <right/>
+      <top style="thin">
+        <color auto="1"/>
+      </top>
+      <bottom style="thin">
+        <color auto="1"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color auto="1"/>
+      </left>
+      <right/>
+      <top style="thin">
+        <color auto="1"/>
+      </top>
+      <bottom style="medium">
+        <color auto="1"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top style="medium">
+        <color indexed="64"/>
+      </top>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom style="medium">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color rgb="FF000000"/>
+      </left>
+      <right style="medium">
+        <color rgb="FF000000"/>
+      </right>
+      <top style="medium">
+        <color rgb="FF000000"/>
+      </top>
+      <bottom style="medium">
+        <color rgb="FF000000"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="medium">
+        <color rgb="FF000000"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
   </borders>
-  <cellStyleXfs count="1">
+  <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="36">
+  <cellXfs count="85">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="2" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
@@ -775,36 +1267,174 @@
     <xf numFmtId="0" fontId="7" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="10" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="6" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="8" fillId="4" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="4" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="4" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="5" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="6" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1" indent="1"/>
     </xf>
-    <xf numFmtId="0" fontId="10" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="4" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="0" xfId="1"/>
+    <xf numFmtId="0" fontId="13" fillId="8" borderId="1" xfId="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="9" fillId="4" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="13" fillId="11" borderId="2" xfId="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="12" borderId="1" xfId="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="10" fillId="4" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
+    <xf numFmtId="0" fontId="14" fillId="9" borderId="3" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="9" borderId="9" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="10" borderId="3" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="10" borderId="9" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="11" borderId="3" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="11" borderId="9" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="3" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="9" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="11" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="10" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="9" borderId="2" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="10" borderId="2" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="13" borderId="0" xfId="1" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="10" borderId="16" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="11" borderId="16" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="0" borderId="0" xfId="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="16" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="17" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="2" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="18" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="13" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="14" borderId="3" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="14" borderId="12" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="14" borderId="14" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="12" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="14" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="2" fontId="0" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="2" fontId="0" fillId="0" borderId="12" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="2" fontId="0" fillId="0" borderId="14" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="2" fontId="0" fillId="0" borderId="11" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="2" fontId="0" fillId="0" borderId="19" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="2" fontId="0" fillId="0" borderId="15" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="15" borderId="20" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="15" borderId="20" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="16" borderId="20" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="17" borderId="20" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="15" borderId="20" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="168" fontId="1" fillId="0" borderId="20" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="0" borderId="21" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="168" fontId="18" fillId="0" borderId="21" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="18" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="168" fontId="18" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
   </cellXfs>
-  <cellStyles count="1">
+  <cellStyles count="2">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
+    <cellStyle name="Normal 2" xfId="1" xr:uid="{219F4CB2-9FAC-4FF4-A885-1E62907124BF}"/>
   </cellStyles>
   <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
@@ -1129,394 +1759,394 @@
       <c r="B1" s="5"/>
       <c r="C1" s="5"/>
       <c r="D1" s="5"/>
-      <c r="E1" s="31" t="s">
+      <c r="E1" s="30" t="s">
         <v>4</v>
       </c>
-      <c r="F1" s="32"/>
-      <c r="G1" s="32"/>
-      <c r="H1" s="32"/>
-      <c r="I1" s="32"/>
-      <c r="J1" s="32"/>
-      <c r="K1" s="32"/>
-      <c r="L1" s="32"/>
-      <c r="M1" s="32"/>
+      <c r="F1" s="31"/>
+      <c r="G1" s="31"/>
+      <c r="H1" s="31"/>
+      <c r="I1" s="31"/>
+      <c r="J1" s="31"/>
+      <c r="K1" s="31"/>
+      <c r="L1" s="31"/>
+      <c r="M1" s="31"/>
       <c r="N1" s="5"/>
       <c r="O1" s="5"/>
       <c r="P1" s="5"/>
       <c r="Q1" s="6"/>
     </row>
     <row r="2" spans="1:17" ht="34" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A2" s="33" t="s">
+      <c r="A2" s="32" t="s">
         <v>11</v>
       </c>
-      <c r="B2" s="33"/>
-      <c r="C2" s="33"/>
-      <c r="D2" s="33"/>
-      <c r="E2" s="33"/>
-      <c r="F2" s="33"/>
-      <c r="G2" s="33"/>
-      <c r="H2" s="33"/>
-      <c r="I2" s="33"/>
-      <c r="J2" s="33"/>
-      <c r="K2" s="33"/>
-      <c r="L2" s="33"/>
-      <c r="M2" s="33"/>
-      <c r="N2" s="33"/>
-      <c r="O2" s="33"/>
-      <c r="P2" s="33"/>
-      <c r="Q2" s="33"/>
+      <c r="B2" s="32"/>
+      <c r="C2" s="32"/>
+      <c r="D2" s="32"/>
+      <c r="E2" s="32"/>
+      <c r="F2" s="32"/>
+      <c r="G2" s="32"/>
+      <c r="H2" s="32"/>
+      <c r="I2" s="32"/>
+      <c r="J2" s="32"/>
+      <c r="K2" s="32"/>
+      <c r="L2" s="32"/>
+      <c r="M2" s="32"/>
+      <c r="N2" s="32"/>
+      <c r="O2" s="32"/>
+      <c r="P2" s="32"/>
+      <c r="Q2" s="32"/>
     </row>
     <row r="3" spans="1:17" ht="13" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A3" s="34" t="s">
+      <c r="A3" s="33" t="s">
         <v>10</v>
       </c>
-      <c r="B3" s="34"/>
-      <c r="C3" s="34"/>
-      <c r="D3" s="34"/>
-      <c r="E3" s="34"/>
-      <c r="F3" s="34"/>
-      <c r="G3" s="34"/>
-      <c r="H3" s="34"/>
-      <c r="I3" s="34"/>
-      <c r="J3" s="34"/>
-      <c r="K3" s="34"/>
-      <c r="L3" s="34"/>
-      <c r="M3" s="34"/>
-      <c r="N3" s="34"/>
-      <c r="O3" s="34"/>
-      <c r="P3" s="34"/>
-      <c r="Q3" s="34"/>
+      <c r="B3" s="33"/>
+      <c r="C3" s="33"/>
+      <c r="D3" s="33"/>
+      <c r="E3" s="33"/>
+      <c r="F3" s="33"/>
+      <c r="G3" s="33"/>
+      <c r="H3" s="33"/>
+      <c r="I3" s="33"/>
+      <c r="J3" s="33"/>
+      <c r="K3" s="33"/>
+      <c r="L3" s="33"/>
+      <c r="M3" s="33"/>
+      <c r="N3" s="33"/>
+      <c r="O3" s="33"/>
+      <c r="P3" s="33"/>
+      <c r="Q3" s="33"/>
     </row>
     <row r="4" spans="1:17" ht="23" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A4" s="34"/>
-      <c r="B4" s="34"/>
-      <c r="C4" s="34"/>
-      <c r="D4" s="34"/>
-      <c r="E4" s="34"/>
-      <c r="F4" s="34"/>
-      <c r="G4" s="34"/>
-      <c r="H4" s="34"/>
-      <c r="I4" s="34"/>
-      <c r="J4" s="34"/>
-      <c r="K4" s="34"/>
-      <c r="L4" s="34"/>
-      <c r="M4" s="34"/>
-      <c r="N4" s="34"/>
-      <c r="O4" s="34"/>
-      <c r="P4" s="34"/>
-      <c r="Q4" s="34"/>
+      <c r="A4" s="33"/>
+      <c r="B4" s="33"/>
+      <c r="C4" s="33"/>
+      <c r="D4" s="33"/>
+      <c r="E4" s="33"/>
+      <c r="F4" s="33"/>
+      <c r="G4" s="33"/>
+      <c r="H4" s="33"/>
+      <c r="I4" s="33"/>
+      <c r="J4" s="33"/>
+      <c r="K4" s="33"/>
+      <c r="L4" s="33"/>
+      <c r="M4" s="33"/>
+      <c r="N4" s="33"/>
+      <c r="O4" s="33"/>
+      <c r="P4" s="33"/>
+      <c r="Q4" s="33"/>
     </row>
     <row r="5" spans="1:17" ht="27" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A5" s="30" t="s">
+      <c r="A5" s="27" t="s">
         <v>12</v>
       </c>
-      <c r="B5" s="30"/>
-      <c r="C5" s="30"/>
-      <c r="D5" s="30"/>
-      <c r="E5" s="30"/>
-      <c r="F5" s="30"/>
-      <c r="G5" s="30"/>
-      <c r="H5" s="30"/>
-      <c r="I5" s="30"/>
-      <c r="J5" s="30"/>
-      <c r="K5" s="30"/>
-      <c r="L5" s="30"/>
-      <c r="M5" s="30"/>
-      <c r="N5" s="30"/>
-      <c r="O5" s="30"/>
-      <c r="P5" s="30"/>
-      <c r="Q5" s="30"/>
+      <c r="B5" s="27"/>
+      <c r="C5" s="27"/>
+      <c r="D5" s="27"/>
+      <c r="E5" s="27"/>
+      <c r="F5" s="27"/>
+      <c r="G5" s="27"/>
+      <c r="H5" s="27"/>
+      <c r="I5" s="27"/>
+      <c r="J5" s="27"/>
+      <c r="K5" s="27"/>
+      <c r="L5" s="27"/>
+      <c r="M5" s="27"/>
+      <c r="N5" s="27"/>
+      <c r="O5" s="27"/>
+      <c r="P5" s="27"/>
+      <c r="Q5" s="27"/>
     </row>
     <row r="6" spans="1:17" ht="158" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A6" s="27" t="s">
+      <c r="A6" s="29" t="s">
         <v>13</v>
       </c>
-      <c r="B6" s="27"/>
-      <c r="C6" s="27"/>
-      <c r="D6" s="27"/>
-      <c r="E6" s="27"/>
-      <c r="F6" s="27"/>
-      <c r="G6" s="27"/>
-      <c r="H6" s="27"/>
-      <c r="I6" s="27"/>
-      <c r="J6" s="27"/>
-      <c r="K6" s="27"/>
-      <c r="L6" s="27"/>
-      <c r="M6" s="27"/>
-      <c r="N6" s="27"/>
-      <c r="O6" s="27"/>
-      <c r="P6" s="27"/>
-      <c r="Q6" s="27"/>
+      <c r="B6" s="29"/>
+      <c r="C6" s="29"/>
+      <c r="D6" s="29"/>
+      <c r="E6" s="29"/>
+      <c r="F6" s="29"/>
+      <c r="G6" s="29"/>
+      <c r="H6" s="29"/>
+      <c r="I6" s="29"/>
+      <c r="J6" s="29"/>
+      <c r="K6" s="29"/>
+      <c r="L6" s="29"/>
+      <c r="M6" s="29"/>
+      <c r="N6" s="29"/>
+      <c r="O6" s="29"/>
+      <c r="P6" s="29"/>
+      <c r="Q6" s="29"/>
     </row>
     <row r="7" spans="1:17" ht="26" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A7" s="30" t="s">
+      <c r="A7" s="27" t="s">
         <v>14</v>
       </c>
-      <c r="B7" s="35"/>
-      <c r="C7" s="35"/>
-      <c r="D7" s="35"/>
-      <c r="E7" s="35"/>
-      <c r="F7" s="35"/>
-      <c r="G7" s="35"/>
-      <c r="H7" s="35"/>
-      <c r="I7" s="35"/>
-      <c r="J7" s="35"/>
-      <c r="K7" s="35"/>
-      <c r="L7" s="35"/>
-      <c r="M7" s="35"/>
-      <c r="N7" s="35"/>
-      <c r="O7" s="35"/>
-      <c r="P7" s="35"/>
-      <c r="Q7" s="35"/>
+      <c r="B7" s="28"/>
+      <c r="C7" s="28"/>
+      <c r="D7" s="28"/>
+      <c r="E7" s="28"/>
+      <c r="F7" s="28"/>
+      <c r="G7" s="28"/>
+      <c r="H7" s="28"/>
+      <c r="I7" s="28"/>
+      <c r="J7" s="28"/>
+      <c r="K7" s="28"/>
+      <c r="L7" s="28"/>
+      <c r="M7" s="28"/>
+      <c r="N7" s="28"/>
+      <c r="O7" s="28"/>
+      <c r="P7" s="28"/>
+      <c r="Q7" s="28"/>
     </row>
     <row r="8" spans="1:17" ht="17.5" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A8" s="27" t="s">
+      <c r="A8" s="29" t="s">
         <v>17</v>
       </c>
-      <c r="B8" s="27"/>
-      <c r="C8" s="27"/>
-      <c r="D8" s="27"/>
-      <c r="E8" s="27"/>
-      <c r="F8" s="27"/>
-      <c r="G8" s="27"/>
-      <c r="H8" s="27"/>
-      <c r="I8" s="27"/>
-      <c r="J8" s="27"/>
-      <c r="K8" s="27"/>
-      <c r="L8" s="27"/>
-      <c r="M8" s="27"/>
-      <c r="N8" s="27"/>
-      <c r="O8" s="27"/>
-      <c r="P8" s="27"/>
-      <c r="Q8" s="27"/>
+      <c r="B8" s="29"/>
+      <c r="C8" s="29"/>
+      <c r="D8" s="29"/>
+      <c r="E8" s="29"/>
+      <c r="F8" s="29"/>
+      <c r="G8" s="29"/>
+      <c r="H8" s="29"/>
+      <c r="I8" s="29"/>
+      <c r="J8" s="29"/>
+      <c r="K8" s="29"/>
+      <c r="L8" s="29"/>
+      <c r="M8" s="29"/>
+      <c r="N8" s="29"/>
+      <c r="O8" s="29"/>
+      <c r="P8" s="29"/>
+      <c r="Q8" s="29"/>
     </row>
     <row r="9" spans="1:17" ht="23" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A9" s="27"/>
-      <c r="B9" s="27"/>
-      <c r="C9" s="27"/>
-      <c r="D9" s="27"/>
-      <c r="E9" s="27"/>
-      <c r="F9" s="27"/>
-      <c r="G9" s="27"/>
-      <c r="H9" s="27"/>
-      <c r="I9" s="27"/>
-      <c r="J9" s="27"/>
-      <c r="K9" s="27"/>
-      <c r="L9" s="27"/>
-      <c r="M9" s="27"/>
-      <c r="N9" s="27"/>
-      <c r="O9" s="27"/>
-      <c r="P9" s="27"/>
-      <c r="Q9" s="27"/>
+      <c r="A9" s="29"/>
+      <c r="B9" s="29"/>
+      <c r="C9" s="29"/>
+      <c r="D9" s="29"/>
+      <c r="E9" s="29"/>
+      <c r="F9" s="29"/>
+      <c r="G9" s="29"/>
+      <c r="H9" s="29"/>
+      <c r="I9" s="29"/>
+      <c r="J9" s="29"/>
+      <c r="K9" s="29"/>
+      <c r="L9" s="29"/>
+      <c r="M9" s="29"/>
+      <c r="N9" s="29"/>
+      <c r="O9" s="29"/>
+      <c r="P9" s="29"/>
+      <c r="Q9" s="29"/>
     </row>
     <row r="10" spans="1:17" ht="30" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A10" s="27"/>
-      <c r="B10" s="27"/>
-      <c r="C10" s="27"/>
-      <c r="D10" s="27"/>
-      <c r="E10" s="27"/>
-      <c r="F10" s="27"/>
-      <c r="G10" s="27"/>
-      <c r="H10" s="27"/>
-      <c r="I10" s="27"/>
-      <c r="J10" s="27"/>
-      <c r="K10" s="27"/>
-      <c r="L10" s="27"/>
-      <c r="M10" s="27"/>
-      <c r="N10" s="27"/>
-      <c r="O10" s="27"/>
-      <c r="P10" s="27"/>
-      <c r="Q10" s="27"/>
+      <c r="A10" s="29"/>
+      <c r="B10" s="29"/>
+      <c r="C10" s="29"/>
+      <c r="D10" s="29"/>
+      <c r="E10" s="29"/>
+      <c r="F10" s="29"/>
+      <c r="G10" s="29"/>
+      <c r="H10" s="29"/>
+      <c r="I10" s="29"/>
+      <c r="J10" s="29"/>
+      <c r="K10" s="29"/>
+      <c r="L10" s="29"/>
+      <c r="M10" s="29"/>
+      <c r="N10" s="29"/>
+      <c r="O10" s="29"/>
+      <c r="P10" s="29"/>
+      <c r="Q10" s="29"/>
     </row>
     <row r="11" spans="1:17" ht="303" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A11" s="27"/>
-      <c r="B11" s="27"/>
-      <c r="C11" s="27"/>
-      <c r="D11" s="27"/>
-      <c r="E11" s="27"/>
-      <c r="F11" s="27"/>
-      <c r="G11" s="27"/>
-      <c r="H11" s="27"/>
-      <c r="I11" s="27"/>
-      <c r="J11" s="27"/>
-      <c r="K11" s="27"/>
-      <c r="L11" s="27"/>
-      <c r="M11" s="27"/>
-      <c r="N11" s="27"/>
-      <c r="O11" s="27"/>
-      <c r="P11" s="27"/>
-      <c r="Q11" s="27"/>
+      <c r="A11" s="29"/>
+      <c r="B11" s="29"/>
+      <c r="C11" s="29"/>
+      <c r="D11" s="29"/>
+      <c r="E11" s="29"/>
+      <c r="F11" s="29"/>
+      <c r="G11" s="29"/>
+      <c r="H11" s="29"/>
+      <c r="I11" s="29"/>
+      <c r="J11" s="29"/>
+      <c r="K11" s="29"/>
+      <c r="L11" s="29"/>
+      <c r="M11" s="29"/>
+      <c r="N11" s="29"/>
+      <c r="O11" s="29"/>
+      <c r="P11" s="29"/>
+      <c r="Q11" s="29"/>
     </row>
     <row r="12" spans="1:17" ht="28" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A12" s="30" t="s">
+      <c r="A12" s="27" t="s">
         <v>15</v>
       </c>
-      <c r="B12" s="30"/>
-      <c r="C12" s="30"/>
-      <c r="D12" s="30"/>
-      <c r="E12" s="30"/>
-      <c r="F12" s="30"/>
-      <c r="G12" s="30"/>
-      <c r="H12" s="30"/>
-      <c r="I12" s="30"/>
-      <c r="J12" s="30"/>
-      <c r="K12" s="30"/>
-      <c r="L12" s="30"/>
-      <c r="M12" s="30"/>
-      <c r="N12" s="30"/>
-      <c r="O12" s="30"/>
-      <c r="P12" s="30"/>
-      <c r="Q12" s="30"/>
+      <c r="B12" s="27"/>
+      <c r="C12" s="27"/>
+      <c r="D12" s="27"/>
+      <c r="E12" s="27"/>
+      <c r="F12" s="27"/>
+      <c r="G12" s="27"/>
+      <c r="H12" s="27"/>
+      <c r="I12" s="27"/>
+      <c r="J12" s="27"/>
+      <c r="K12" s="27"/>
+      <c r="L12" s="27"/>
+      <c r="M12" s="27"/>
+      <c r="N12" s="27"/>
+      <c r="O12" s="27"/>
+      <c r="P12" s="27"/>
+      <c r="Q12" s="27"/>
     </row>
     <row r="15" spans="1:17" ht="191.5" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A15" s="29" t="s">
+      <c r="A15" s="35" t="s">
         <v>18</v>
       </c>
-      <c r="B15" s="29"/>
-      <c r="C15" s="29"/>
-      <c r="D15" s="29"/>
-      <c r="E15" s="29"/>
-      <c r="F15" s="29"/>
-      <c r="G15" s="29"/>
-      <c r="H15" s="29"/>
-      <c r="I15" s="29"/>
-      <c r="J15" s="29"/>
-      <c r="K15" s="29"/>
-      <c r="L15" s="29"/>
-      <c r="M15" s="29"/>
-      <c r="N15" s="29"/>
-      <c r="O15" s="29"/>
-      <c r="P15" s="29"/>
+      <c r="B15" s="35"/>
+      <c r="C15" s="35"/>
+      <c r="D15" s="35"/>
+      <c r="E15" s="35"/>
+      <c r="F15" s="35"/>
+      <c r="G15" s="35"/>
+      <c r="H15" s="35"/>
+      <c r="I15" s="35"/>
+      <c r="J15" s="35"/>
+      <c r="K15" s="35"/>
+      <c r="L15" s="35"/>
+      <c r="M15" s="35"/>
+      <c r="N15" s="35"/>
+      <c r="O15" s="35"/>
+      <c r="P15" s="35"/>
     </row>
     <row r="16" spans="1:17" ht="28" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A16" s="30" t="s">
+      <c r="A16" s="27" t="s">
         <v>5</v>
       </c>
-      <c r="B16" s="30"/>
-      <c r="C16" s="30"/>
-      <c r="D16" s="30"/>
-      <c r="E16" s="30"/>
-      <c r="F16" s="30"/>
-      <c r="G16" s="30"/>
-      <c r="H16" s="30"/>
-      <c r="I16" s="30"/>
-      <c r="J16" s="30"/>
-      <c r="K16" s="30"/>
-      <c r="L16" s="30"/>
-      <c r="M16" s="30"/>
-      <c r="N16" s="30"/>
-      <c r="O16" s="30"/>
-      <c r="P16" s="30"/>
+      <c r="B16" s="27"/>
+      <c r="C16" s="27"/>
+      <c r="D16" s="27"/>
+      <c r="E16" s="27"/>
+      <c r="F16" s="27"/>
+      <c r="G16" s="27"/>
+      <c r="H16" s="27"/>
+      <c r="I16" s="27"/>
+      <c r="J16" s="27"/>
+      <c r="K16" s="27"/>
+      <c r="L16" s="27"/>
+      <c r="M16" s="27"/>
+      <c r="N16" s="27"/>
+      <c r="O16" s="27"/>
+      <c r="P16" s="27"/>
     </row>
     <row r="17" spans="1:17" ht="24" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A17" s="29" t="s">
+      <c r="A17" s="35" t="s">
         <v>16</v>
       </c>
-      <c r="B17" s="29"/>
-      <c r="C17" s="29"/>
-      <c r="D17" s="29"/>
-      <c r="E17" s="29"/>
-      <c r="F17" s="29"/>
-      <c r="G17" s="29"/>
-      <c r="H17" s="29"/>
-      <c r="I17" s="29"/>
-      <c r="J17" s="29"/>
-      <c r="K17" s="29"/>
-      <c r="L17" s="29"/>
-      <c r="M17" s="29"/>
-      <c r="N17" s="29"/>
-      <c r="O17" s="29"/>
-      <c r="P17" s="29"/>
+      <c r="B17" s="35"/>
+      <c r="C17" s="35"/>
+      <c r="D17" s="35"/>
+      <c r="E17" s="35"/>
+      <c r="F17" s="35"/>
+      <c r="G17" s="35"/>
+      <c r="H17" s="35"/>
+      <c r="I17" s="35"/>
+      <c r="J17" s="35"/>
+      <c r="K17" s="35"/>
+      <c r="L17" s="35"/>
+      <c r="M17" s="35"/>
+      <c r="N17" s="35"/>
+      <c r="O17" s="35"/>
+      <c r="P17" s="35"/>
     </row>
     <row r="18" spans="1:17" ht="53.5" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A18" s="29"/>
-      <c r="B18" s="29"/>
-      <c r="C18" s="29"/>
-      <c r="D18" s="29"/>
-      <c r="E18" s="29"/>
-      <c r="F18" s="29"/>
-      <c r="G18" s="29"/>
-      <c r="H18" s="29"/>
-      <c r="I18" s="29"/>
-      <c r="J18" s="29"/>
-      <c r="K18" s="29"/>
-      <c r="L18" s="29"/>
-      <c r="M18" s="29"/>
-      <c r="N18" s="29"/>
-      <c r="O18" s="29"/>
-      <c r="P18" s="29"/>
+      <c r="A18" s="35"/>
+      <c r="B18" s="35"/>
+      <c r="C18" s="35"/>
+      <c r="D18" s="35"/>
+      <c r="E18" s="35"/>
+      <c r="F18" s="35"/>
+      <c r="G18" s="35"/>
+      <c r="H18" s="35"/>
+      <c r="I18" s="35"/>
+      <c r="J18" s="35"/>
+      <c r="K18" s="35"/>
+      <c r="L18" s="35"/>
+      <c r="M18" s="35"/>
+      <c r="N18" s="35"/>
+      <c r="O18" s="35"/>
+      <c r="P18" s="35"/>
     </row>
     <row r="19" spans="1:17" ht="24" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A19" s="29"/>
-      <c r="B19" s="29"/>
-      <c r="C19" s="29"/>
-      <c r="D19" s="29"/>
-      <c r="E19" s="29"/>
-      <c r="F19" s="29"/>
-      <c r="G19" s="29"/>
-      <c r="H19" s="29"/>
-      <c r="I19" s="29"/>
-      <c r="J19" s="29"/>
-      <c r="K19" s="29"/>
-      <c r="L19" s="29"/>
-      <c r="M19" s="29"/>
-      <c r="N19" s="29"/>
-      <c r="O19" s="29"/>
-      <c r="P19" s="29"/>
+      <c r="A19" s="35"/>
+      <c r="B19" s="35"/>
+      <c r="C19" s="35"/>
+      <c r="D19" s="35"/>
+      <c r="E19" s="35"/>
+      <c r="F19" s="35"/>
+      <c r="G19" s="35"/>
+      <c r="H19" s="35"/>
+      <c r="I19" s="35"/>
+      <c r="J19" s="35"/>
+      <c r="K19" s="35"/>
+      <c r="L19" s="35"/>
+      <c r="M19" s="35"/>
+      <c r="N19" s="35"/>
+      <c r="O19" s="35"/>
+      <c r="P19" s="35"/>
     </row>
     <row r="20" spans="1:17" ht="18.5" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A20" s="29"/>
-      <c r="B20" s="29"/>
-      <c r="C20" s="29"/>
-      <c r="D20" s="29"/>
-      <c r="E20" s="29"/>
-      <c r="F20" s="29"/>
-      <c r="G20" s="29"/>
-      <c r="H20" s="29"/>
-      <c r="I20" s="29"/>
-      <c r="J20" s="29"/>
-      <c r="K20" s="29"/>
-      <c r="L20" s="29"/>
-      <c r="M20" s="29"/>
-      <c r="N20" s="29"/>
-      <c r="O20" s="29"/>
-      <c r="P20" s="29"/>
+      <c r="A20" s="35"/>
+      <c r="B20" s="35"/>
+      <c r="C20" s="35"/>
+      <c r="D20" s="35"/>
+      <c r="E20" s="35"/>
+      <c r="F20" s="35"/>
+      <c r="G20" s="35"/>
+      <c r="H20" s="35"/>
+      <c r="I20" s="35"/>
+      <c r="J20" s="35"/>
+      <c r="K20" s="35"/>
+      <c r="L20" s="35"/>
+      <c r="M20" s="35"/>
+      <c r="N20" s="35"/>
+      <c r="O20" s="35"/>
+      <c r="P20" s="35"/>
     </row>
     <row r="21" spans="1:17" ht="19" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A21" s="27"/>
-      <c r="B21" s="27"/>
-      <c r="C21" s="27"/>
-      <c r="D21" s="27"/>
-      <c r="E21" s="27"/>
-      <c r="F21" s="27"/>
-      <c r="G21" s="27"/>
-      <c r="H21" s="27"/>
-      <c r="I21" s="27"/>
-      <c r="J21" s="27"/>
-      <c r="K21" s="27"/>
-      <c r="L21" s="27"/>
-      <c r="M21" s="27"/>
-      <c r="N21" s="27"/>
-      <c r="O21" s="27"/>
-      <c r="P21" s="27"/>
+      <c r="A21" s="29"/>
+      <c r="B21" s="29"/>
+      <c r="C21" s="29"/>
+      <c r="D21" s="29"/>
+      <c r="E21" s="29"/>
+      <c r="F21" s="29"/>
+      <c r="G21" s="29"/>
+      <c r="H21" s="29"/>
+      <c r="I21" s="29"/>
+      <c r="J21" s="29"/>
+      <c r="K21" s="29"/>
+      <c r="L21" s="29"/>
+      <c r="M21" s="29"/>
+      <c r="N21" s="29"/>
+      <c r="O21" s="29"/>
+      <c r="P21" s="29"/>
     </row>
     <row r="22" spans="1:17" ht="20" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A22" s="27"/>
-      <c r="B22" s="27"/>
-      <c r="C22" s="27"/>
-      <c r="D22" s="27"/>
-      <c r="E22" s="27"/>
-      <c r="F22" s="27"/>
-      <c r="G22" s="27"/>
-      <c r="H22" s="27"/>
-      <c r="I22" s="27"/>
-      <c r="J22" s="27"/>
-      <c r="K22" s="27"/>
-      <c r="L22" s="27"/>
-      <c r="M22" s="27"/>
-      <c r="N22" s="27"/>
-      <c r="O22" s="27"/>
-      <c r="P22" s="27"/>
+      <c r="A22" s="29"/>
+      <c r="B22" s="29"/>
+      <c r="C22" s="29"/>
+      <c r="D22" s="29"/>
+      <c r="E22" s="29"/>
+      <c r="F22" s="29"/>
+      <c r="G22" s="29"/>
+      <c r="H22" s="29"/>
+      <c r="I22" s="29"/>
+      <c r="J22" s="29"/>
+      <c r="K22" s="29"/>
+      <c r="L22" s="29"/>
+      <c r="M22" s="29"/>
+      <c r="N22" s="29"/>
+      <c r="O22" s="29"/>
+      <c r="P22" s="29"/>
       <c r="Q22" s="26"/>
     </row>
     <row r="23" spans="1:17" ht="16.5" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
@@ -1544,11 +2174,11 @@
       <c r="D24" s="9"/>
       <c r="E24" s="9"/>
       <c r="F24" s="9"/>
-      <c r="G24" s="28" t="s">
+      <c r="G24" s="34" t="s">
         <v>6</v>
       </c>
-      <c r="H24" s="28"/>
-      <c r="I24" s="28"/>
+      <c r="H24" s="34"/>
+      <c r="I24" s="34"/>
       <c r="J24" s="9"/>
       <c r="K24" s="9"/>
       <c r="L24" s="9"/>
@@ -1558,9 +2188,9 @@
       <c r="P24" s="9"/>
     </row>
     <row r="25" spans="1:17" hidden="1" x14ac:dyDescent="0.35">
-      <c r="G25" s="28"/>
-      <c r="H25" s="28"/>
-      <c r="I25" s="28"/>
+      <c r="G25" s="34"/>
+      <c r="H25" s="34"/>
+      <c r="I25" s="34"/>
     </row>
     <row r="35" spans="1:17" ht="15.5" hidden="1" x14ac:dyDescent="0.35">
       <c r="Q35" s="8"/>
@@ -1670,6 +2300,11 @@
     <row r="71" ht="14.5" hidden="1" customHeight="1" x14ac:dyDescent="0.35"/>
   </sheetData>
   <mergeCells count="13">
+    <mergeCell ref="A21:P22"/>
+    <mergeCell ref="G24:I25"/>
+    <mergeCell ref="A15:P15"/>
+    <mergeCell ref="A16:P16"/>
+    <mergeCell ref="A17:P20"/>
     <mergeCell ref="A7:Q7"/>
     <mergeCell ref="A8:Q11"/>
     <mergeCell ref="A12:Q12"/>
@@ -1678,11 +2313,6 @@
     <mergeCell ref="A3:Q4"/>
     <mergeCell ref="A5:Q5"/>
     <mergeCell ref="A6:Q6"/>
-    <mergeCell ref="A21:P22"/>
-    <mergeCell ref="G24:I25"/>
-    <mergeCell ref="A15:P15"/>
-    <mergeCell ref="A16:P16"/>
-    <mergeCell ref="A17:P20"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
@@ -2120,4 +2750,2401 @@
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{3673BA12-1B53-4038-BC7A-55A8B8949BFD}">
+  <dimension ref="A1:U20"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetData>
+    <row r="1" spans="1:21" ht="72.5" x14ac:dyDescent="0.35">
+      <c r="A1" s="37" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="50" t="s">
+        <v>19</v>
+      </c>
+      <c r="C1" s="50" t="s">
+        <v>19</v>
+      </c>
+      <c r="D1" s="50" t="s">
+        <v>19</v>
+      </c>
+      <c r="E1" s="50" t="s">
+        <v>19</v>
+      </c>
+      <c r="F1" s="50" t="s">
+        <v>19</v>
+      </c>
+      <c r="G1" s="51" t="s">
+        <v>20</v>
+      </c>
+      <c r="H1" s="51" t="s">
+        <v>20</v>
+      </c>
+      <c r="I1" s="51" t="s">
+        <v>20</v>
+      </c>
+      <c r="J1" s="51" t="s">
+        <v>20</v>
+      </c>
+      <c r="K1" s="51" t="s">
+        <v>20</v>
+      </c>
+      <c r="L1" s="38" t="s">
+        <v>21</v>
+      </c>
+      <c r="M1" s="38" t="s">
+        <v>21</v>
+      </c>
+      <c r="N1" s="38" t="s">
+        <v>21</v>
+      </c>
+      <c r="O1" s="38" t="s">
+        <v>21</v>
+      </c>
+      <c r="P1" s="38" t="s">
+        <v>21</v>
+      </c>
+      <c r="Q1" s="52" t="s">
+        <v>22</v>
+      </c>
+      <c r="R1" s="52" t="s">
+        <v>22</v>
+      </c>
+      <c r="S1" s="52" t="s">
+        <v>22</v>
+      </c>
+      <c r="T1" s="52" t="s">
+        <v>22</v>
+      </c>
+      <c r="U1" s="52" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="2" spans="1:21" ht="43.5" x14ac:dyDescent="0.35">
+      <c r="A2" s="39"/>
+      <c r="B2" s="40" t="s">
+        <v>23</v>
+      </c>
+      <c r="C2" s="40" t="s">
+        <v>24</v>
+      </c>
+      <c r="D2" s="40" t="s">
+        <v>25</v>
+      </c>
+      <c r="E2" s="40" t="s">
+        <v>26</v>
+      </c>
+      <c r="F2" s="41" t="s">
+        <v>27</v>
+      </c>
+      <c r="G2" s="42" t="s">
+        <v>23</v>
+      </c>
+      <c r="H2" s="42" t="s">
+        <v>24</v>
+      </c>
+      <c r="I2" s="42" t="s">
+        <v>25</v>
+      </c>
+      <c r="J2" s="53" t="s">
+        <v>26</v>
+      </c>
+      <c r="K2" s="43" t="s">
+        <v>27</v>
+      </c>
+      <c r="L2" s="44" t="s">
+        <v>23</v>
+      </c>
+      <c r="M2" s="44" t="s">
+        <v>24</v>
+      </c>
+      <c r="N2" s="54" t="s">
+        <v>25</v>
+      </c>
+      <c r="O2" s="54" t="s">
+        <v>26</v>
+      </c>
+      <c r="P2" s="45" t="s">
+        <v>27</v>
+      </c>
+      <c r="Q2" s="55" t="s">
+        <v>23</v>
+      </c>
+      <c r="R2" s="55" t="s">
+        <v>28</v>
+      </c>
+      <c r="S2" s="55" t="s">
+        <v>25</v>
+      </c>
+      <c r="T2" s="55" t="s">
+        <v>26</v>
+      </c>
+      <c r="U2" s="55" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="3" spans="1:21" x14ac:dyDescent="0.35">
+      <c r="A3" s="36" t="s">
+        <v>29</v>
+      </c>
+      <c r="B3" s="46">
+        <v>1.7709494061731681</v>
+      </c>
+      <c r="C3" s="46">
+        <v>2.668645377141138</v>
+      </c>
+      <c r="D3" s="46">
+        <v>5.7663953494565663E-2</v>
+      </c>
+      <c r="E3" s="46">
+        <v>25.412554751205519</v>
+      </c>
+      <c r="F3" s="47">
+        <v>0.79790850389123436</v>
+      </c>
+      <c r="G3" s="46">
+        <v>1.8562963655068148</v>
+      </c>
+      <c r="H3" s="46">
+        <v>2.7972547929069762</v>
+      </c>
+      <c r="I3" s="46">
+        <v>4.649456861934396E-3</v>
+      </c>
+      <c r="J3" s="56">
+        <v>0.10969913124770765</v>
+      </c>
+      <c r="K3" s="47">
+        <v>0.77155671628335842</v>
+      </c>
+      <c r="L3" s="46">
+        <v>1.7709494061731681</v>
+      </c>
+      <c r="M3" s="46">
+        <v>2.668645377141138</v>
+      </c>
+      <c r="N3" s="56">
+        <v>4.435688730351205E-3</v>
+      </c>
+      <c r="O3" s="56">
+        <v>0.19548119039388856</v>
+      </c>
+      <c r="P3" s="47">
+        <v>0.73392015952255707</v>
+      </c>
+      <c r="Q3" s="36">
+        <v>1.7709494061731681</v>
+      </c>
+      <c r="R3" s="36">
+        <v>0.58334737489988697</v>
+      </c>
+      <c r="S3" s="36">
+        <v>4.435688730351205E-3</v>
+      </c>
+      <c r="T3" s="36">
+        <v>0.19548119039388856</v>
+      </c>
+      <c r="U3" s="36">
+        <v>5.711748379119308E-3</v>
+      </c>
+    </row>
+    <row r="4" spans="1:21" x14ac:dyDescent="0.35">
+      <c r="A4" s="36" t="s">
+        <v>30</v>
+      </c>
+      <c r="B4" s="46">
+        <v>7.8220577847384464E-5</v>
+      </c>
+      <c r="C4" s="46">
+        <v>9.0661426286863534E-5</v>
+      </c>
+      <c r="D4" s="46">
+        <v>2.6175296172958929E-6</v>
+      </c>
+      <c r="E4" s="46">
+        <v>3.064622430685465E-5</v>
+      </c>
+      <c r="F4" s="47">
+        <v>1.8200642681422206E-2</v>
+      </c>
+      <c r="G4" s="46">
+        <v>8.199024424966805E-5</v>
+      </c>
+      <c r="H4" s="46">
+        <v>9.5030651650085892E-5</v>
+      </c>
+      <c r="I4" s="46">
+        <v>2.1105197099605442E-7</v>
+      </c>
+      <c r="J4" s="56">
+        <v>1.3229146834695386E-7</v>
+      </c>
+      <c r="K4" s="47">
+        <v>2.1823946459154087E-2</v>
+      </c>
+      <c r="L4" s="46">
+        <v>7.8220577847384464E-5</v>
+      </c>
+      <c r="M4" s="46">
+        <v>9.0661426286863534E-5</v>
+      </c>
+      <c r="N4" s="56">
+        <v>2.0134843209968409E-7</v>
+      </c>
+      <c r="O4" s="56">
+        <v>2.3574018697580496E-7</v>
+      </c>
+      <c r="P4" s="47">
+        <v>1.8199338311173801E-2</v>
+      </c>
+      <c r="Q4" s="36">
+        <v>7.8220577847384464E-5</v>
+      </c>
+      <c r="R4" s="36">
+        <v>5.8272729005051103E-5</v>
+      </c>
+      <c r="S4" s="36">
+        <v>2.0134843209968409E-7</v>
+      </c>
+      <c r="T4" s="36">
+        <v>2.3574018697580496E-7</v>
+      </c>
+      <c r="U4" s="36">
+        <v>1.1116888316618192E-7</v>
+      </c>
+    </row>
+    <row r="5" spans="1:21" x14ac:dyDescent="0.35">
+      <c r="A5" s="36" t="s">
+        <v>31</v>
+      </c>
+      <c r="B5" s="46">
+        <v>7.9090931108826291E-4</v>
+      </c>
+      <c r="C5" s="46">
+        <v>4.9455725746545018E-4</v>
+      </c>
+      <c r="D5" s="46">
+        <v>2.0709323842504656E-5</v>
+      </c>
+      <c r="E5" s="46">
+        <v>2.9334816005991516E-4</v>
+      </c>
+      <c r="F5" s="47">
+        <v>1.7031645445422603E-5</v>
+      </c>
+      <c r="G5" s="46">
+        <v>8.2902542246601047E-4</v>
+      </c>
+      <c r="H5" s="46">
+        <v>5.1839134216258038E-4</v>
+      </c>
+      <c r="I5" s="46">
+        <v>1.6697971958275304E-6</v>
+      </c>
+      <c r="J5" s="56">
+        <v>1.2663047311352917E-6</v>
+      </c>
+      <c r="K5" s="47">
+        <v>1.4186964570181255E-6</v>
+      </c>
+      <c r="L5" s="46">
+        <v>7.9090931108826291E-4</v>
+      </c>
+      <c r="M5" s="46">
+        <v>4.9455725746545018E-4</v>
+      </c>
+      <c r="N5" s="56">
+        <v>1.5930249109618967E-6</v>
+      </c>
+      <c r="O5" s="56">
+        <v>2.2565243081531931E-6</v>
+      </c>
+      <c r="P5" s="47">
+        <v>1.3534577885820813E-6</v>
+      </c>
+      <c r="Q5" s="36">
+        <v>7.9090931108826291E-4</v>
+      </c>
+      <c r="R5" s="36">
+        <v>3.1401530086576287E-4</v>
+      </c>
+      <c r="S5" s="36">
+        <v>1.5930249109618967E-6</v>
+      </c>
+      <c r="T5" s="36">
+        <v>2.2565243081531931E-6</v>
+      </c>
+      <c r="U5" s="36">
+        <v>1.3429122019173875E-6</v>
+      </c>
+    </row>
+    <row r="6" spans="1:21" x14ac:dyDescent="0.35">
+      <c r="A6" s="36" t="s">
+        <v>32</v>
+      </c>
+      <c r="B6" s="46">
+        <v>1.4653687857214052E-6</v>
+      </c>
+      <c r="C6" s="46">
+        <v>9.980146094968135E-6</v>
+      </c>
+      <c r="D6" s="46">
+        <v>5.6335826541772404E-8</v>
+      </c>
+      <c r="E6" s="46">
+        <v>7.131075534057526E-6</v>
+      </c>
+      <c r="F6" s="47">
+        <v>2.6898590332552826E-5</v>
+      </c>
+      <c r="G6" s="46">
+        <v>1.5359889681658103E-6</v>
+      </c>
+      <c r="H6" s="46">
+        <v>1.0461116991111177E-5</v>
+      </c>
+      <c r="I6" s="46">
+        <v>4.5423697026266912E-9</v>
+      </c>
+      <c r="J6" s="56">
+        <v>3.0782925943751647E-8</v>
+      </c>
+      <c r="K6" s="47">
+        <v>2.8255169667100004E-5</v>
+      </c>
+      <c r="L6" s="46">
+        <v>1.4653687857214052E-6</v>
+      </c>
+      <c r="M6" s="46">
+        <v>9.980146094968135E-6</v>
+      </c>
+      <c r="N6" s="56">
+        <v>4.3335251185978782E-9</v>
+      </c>
+      <c r="O6" s="56">
+        <v>5.4854427185057882E-8</v>
+      </c>
+      <c r="P6" s="47">
+        <v>2.6876273188840458E-5</v>
+      </c>
+      <c r="Q6" s="36">
+        <v>1.4653687857214052E-6</v>
+      </c>
+      <c r="R6" s="36">
+        <v>2.2939876092841725E-7</v>
+      </c>
+      <c r="S6" s="36">
+        <v>4.3335251185978782E-9</v>
+      </c>
+      <c r="T6" s="36">
+        <v>5.4854427185057882E-8</v>
+      </c>
+      <c r="U6" s="36">
+        <v>1.9611200149488022E-9</v>
+      </c>
+    </row>
+    <row r="7" spans="1:21" x14ac:dyDescent="0.35">
+      <c r="A7" s="36" t="s">
+        <v>33</v>
+      </c>
+      <c r="B7" s="46">
+        <v>4.3737654181269636E-3</v>
+      </c>
+      <c r="C7" s="46">
+        <v>3.615106069735773E-3</v>
+      </c>
+      <c r="D7" s="46">
+        <v>1.197632792036769E-4</v>
+      </c>
+      <c r="E7" s="46">
+        <v>1.8661039926854084E-2</v>
+      </c>
+      <c r="F7" s="47">
+        <v>2.0050709279814273E-4</v>
+      </c>
+      <c r="G7" s="46">
+        <v>4.5845492936993472E-3</v>
+      </c>
+      <c r="H7" s="46">
+        <v>3.7893280490001479E-3</v>
+      </c>
+      <c r="I7" s="46">
+        <v>9.6565387309730235E-6</v>
+      </c>
+      <c r="J7" s="56">
+        <v>8.055466631341223E-5</v>
+      </c>
+      <c r="K7" s="47">
+        <v>1.7550340284880775E-5</v>
+      </c>
+      <c r="L7" s="46">
+        <v>4.3737654181269636E-3</v>
+      </c>
+      <c r="M7" s="46">
+        <v>3.615106069735773E-3</v>
+      </c>
+      <c r="N7" s="56">
+        <v>9.2125599387443775E-6</v>
+      </c>
+      <c r="O7" s="56">
+        <v>1.4354646097580062E-4</v>
+      </c>
+      <c r="P7" s="47">
+        <v>1.6741685547534787E-5</v>
+      </c>
+      <c r="Q7" s="36">
+        <v>4.3737654181269636E-3</v>
+      </c>
+      <c r="R7" s="36">
+        <v>1.6907364209389965E-3</v>
+      </c>
+      <c r="S7" s="36">
+        <v>9.2125599387443775E-6</v>
+      </c>
+      <c r="T7" s="36">
+        <v>1.4354646097580062E-4</v>
+      </c>
+      <c r="U7" s="36">
+        <v>1.6326891285836631E-5</v>
+      </c>
+    </row>
+    <row r="8" spans="1:21" x14ac:dyDescent="0.35">
+      <c r="A8" s="36" t="s">
+        <v>34</v>
+      </c>
+      <c r="B8" s="46">
+        <v>0.19976665986922368</v>
+      </c>
+      <c r="C8" s="46">
+        <v>9.1455140742736279E-2</v>
+      </c>
+      <c r="D8" s="46">
+        <v>5.3663067951629203E-3</v>
+      </c>
+      <c r="E8" s="46">
+        <v>0.11113014927192315</v>
+      </c>
+      <c r="F8" s="47">
+        <v>1.1594619391389012E-2</v>
+      </c>
+      <c r="G8" s="46">
+        <v>0.20939396877858385</v>
+      </c>
+      <c r="H8" s="46">
+        <v>9.5862617405036835E-2</v>
+      </c>
+      <c r="I8" s="46">
+        <v>4.3268646077773319E-4</v>
+      </c>
+      <c r="J8" s="56">
+        <v>4.7971882205112532E-4</v>
+      </c>
+      <c r="K8" s="47">
+        <v>9.735441260104922E-4</v>
+      </c>
+      <c r="L8" s="46">
+        <v>0.19976665986922368</v>
+      </c>
+      <c r="M8" s="46">
+        <v>9.1455140742736279E-2</v>
+      </c>
+      <c r="N8" s="56">
+        <v>4.1279283039714779E-4</v>
+      </c>
+      <c r="O8" s="56">
+        <v>8.5484730209171638E-4</v>
+      </c>
+      <c r="P8" s="47">
+        <v>9.295089132124487E-4</v>
+      </c>
+      <c r="Q8" s="36">
+        <v>0.19976665986922368</v>
+      </c>
+      <c r="R8" s="36">
+        <v>4.1364241535403787E-2</v>
+      </c>
+      <c r="S8" s="36">
+        <v>4.1279283039714779E-4</v>
+      </c>
+      <c r="T8" s="36">
+        <v>8.5484730209171638E-4</v>
+      </c>
+      <c r="U8" s="36">
+        <v>9.0356095872703393E-4</v>
+      </c>
+    </row>
+    <row r="9" spans="1:21" ht="15" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="A9" s="36" t="s">
+        <v>35</v>
+      </c>
+      <c r="B9" s="48">
+        <v>0.14887591293122765</v>
+      </c>
+      <c r="C9" s="48">
+        <v>0.19170924993024219</v>
+      </c>
+      <c r="D9" s="48">
+        <v>6.837971790117932E-3</v>
+      </c>
+      <c r="E9" s="48">
+        <v>0.17013866179834605</v>
+      </c>
+      <c r="F9" s="49">
+        <v>5.595443090609698E-3</v>
+      </c>
+      <c r="G9" s="48">
+        <v>0.15605065572309407</v>
+      </c>
+      <c r="H9" s="48">
+        <v>0.20094824992688037</v>
+      </c>
+      <c r="I9" s="48">
+        <v>5.5134712302155713E-4</v>
+      </c>
+      <c r="J9" s="57">
+        <v>7.344426238782908E-4</v>
+      </c>
+      <c r="K9" s="49">
+        <v>4.7602337195748419E-4</v>
+      </c>
+      <c r="L9" s="48">
+        <v>0.14887591293122765</v>
+      </c>
+      <c r="M9" s="48">
+        <v>0.19170924993024219</v>
+      </c>
+      <c r="N9" s="57">
+        <v>5.2599783000907173E-4</v>
+      </c>
+      <c r="O9" s="57">
+        <v>1.3087589369103539E-3</v>
+      </c>
+      <c r="P9" s="49">
+        <v>4.5407987152537251E-4</v>
+      </c>
+      <c r="Q9" s="36">
+        <v>0.14887591293122765</v>
+      </c>
+      <c r="R9" s="36">
+        <v>7.1996879817882539E-2</v>
+      </c>
+      <c r="S9" s="36">
+        <v>5.2599783000907173E-4</v>
+      </c>
+      <c r="T9" s="36">
+        <v>1.3087589369103539E-3</v>
+      </c>
+      <c r="U9" s="36">
+        <v>4.4796264413187186E-4</v>
+      </c>
+    </row>
+    <row r="10" spans="1:21" x14ac:dyDescent="0.35">
+      <c r="A10" s="36" t="s">
+        <v>36</v>
+      </c>
+      <c r="B10" s="36">
+        <v>2.7490001309265955</v>
+      </c>
+      <c r="C10" s="36">
+        <v>3.5593597468191671</v>
+      </c>
+      <c r="D10" s="36">
+        <v>7.7236404682858778E-2</v>
+      </c>
+      <c r="E10" s="36">
+        <v>0.8083036506423491</v>
+      </c>
+      <c r="F10" s="36">
+        <v>5.046569853188209E-2</v>
+      </c>
+      <c r="G10" s="36">
+        <v>2.881482064947154</v>
+      </c>
+      <c r="H10" s="36">
+        <v>3.7308951563044288</v>
+      </c>
+      <c r="I10" s="36">
+        <v>6.2275877733166951E-3</v>
+      </c>
+      <c r="J10" s="36">
+        <v>3.4892284198860387E-3</v>
+      </c>
+      <c r="K10" s="36">
+        <v>4.1773509024613156E-3</v>
+      </c>
+      <c r="L10" s="36">
+        <v>2.7490001309265955</v>
+      </c>
+      <c r="M10" s="36">
+        <v>3.5593597468191671</v>
+      </c>
+      <c r="N10" s="36">
+        <v>5.941261898681445E-3</v>
+      </c>
+      <c r="O10" s="36">
+        <v>6.2177203895565298E-3</v>
+      </c>
+      <c r="P10" s="36">
+        <v>3.9851622096092592E-3</v>
+      </c>
+      <c r="Q10" s="36">
+        <v>2.7490001309265955</v>
+      </c>
+      <c r="R10" s="36">
+        <v>1.3574294325226137</v>
+      </c>
+      <c r="S10" s="36">
+        <v>5.941261898681445E-3</v>
+      </c>
+      <c r="T10" s="36">
+        <v>6.2177203895565298E-3</v>
+      </c>
+      <c r="U10" s="36">
+        <v>3.9660184242227689E-3</v>
+      </c>
+    </row>
+    <row r="11" spans="1:21" x14ac:dyDescent="0.35">
+      <c r="A11" s="36" t="s">
+        <v>37</v>
+      </c>
+      <c r="B11" s="36">
+        <v>0.14084532701478866</v>
+      </c>
+      <c r="C11" s="36">
+        <v>0.22035233640855748</v>
+      </c>
+      <c r="D11" s="36">
+        <v>3.4970872804044395E-3</v>
+      </c>
+      <c r="E11" s="36">
+        <v>4.7008515055234235E-2</v>
+      </c>
+      <c r="F11" s="36">
+        <v>1.8373964376244105E-3</v>
+      </c>
+      <c r="G11" s="36">
+        <v>0.14763305361791101</v>
+      </c>
+      <c r="H11" s="36">
+        <v>0.230971726114994</v>
+      </c>
+      <c r="I11" s="36">
+        <v>2.8197089285930145E-4</v>
+      </c>
+      <c r="J11" s="36">
+        <v>2.0292305568212713E-4</v>
+      </c>
+      <c r="K11" s="36">
+        <v>1.5041163986852823E-4</v>
+      </c>
+      <c r="L11" s="36">
+        <v>0.14084532701478866</v>
+      </c>
+      <c r="M11" s="36">
+        <v>0.22035233640855748</v>
+      </c>
+      <c r="N11" s="36">
+        <v>2.6900671387726461E-4</v>
+      </c>
+      <c r="O11" s="36">
+        <v>3.616039619633402E-4</v>
+      </c>
+      <c r="P11" s="36">
+        <v>1.4349542179957264E-4</v>
+      </c>
+      <c r="Q11" s="36">
+        <v>0.14084532701478866</v>
+      </c>
+      <c r="R11" s="36">
+        <v>7.4358583648173299E-2</v>
+      </c>
+      <c r="S11" s="36">
+        <v>2.6900671387726461E-4</v>
+      </c>
+      <c r="T11" s="36">
+        <v>3.616039619633402E-4</v>
+      </c>
+      <c r="U11" s="36">
+        <v>1.4335946782196063E-4</v>
+      </c>
+    </row>
+    <row r="12" spans="1:21" x14ac:dyDescent="0.35">
+      <c r="A12" s="36" t="s">
+        <v>38</v>
+      </c>
+      <c r="B12" s="36">
+        <v>0.18554040818080225</v>
+      </c>
+      <c r="C12" s="36">
+        <v>0.28794463148072125</v>
+      </c>
+      <c r="D12" s="36">
+        <v>4.6775492778877333E-3</v>
+      </c>
+      <c r="E12" s="36">
+        <v>0.10678213371068793</v>
+      </c>
+      <c r="F12" s="36">
+        <v>2.6382994703037055E-3</v>
+      </c>
+      <c r="G12" s="36">
+        <v>0.19448211459915418</v>
+      </c>
+      <c r="H12" s="36">
+        <v>0.30182148119063557</v>
+      </c>
+      <c r="I12" s="36">
+        <v>3.7715179534405266E-4</v>
+      </c>
+      <c r="J12" s="36">
+        <v>4.6094961390229136E-4</v>
+      </c>
+      <c r="K12" s="36">
+        <v>2.1713112654839353E-4</v>
+      </c>
+      <c r="L12" s="36">
+        <v>0.18554040818080225</v>
+      </c>
+      <c r="M12" s="36">
+        <v>0.28794463148072125</v>
+      </c>
+      <c r="N12" s="36">
+        <v>3.5981148291444105E-4</v>
+      </c>
+      <c r="O12" s="36">
+        <v>8.2140102854375322E-4</v>
+      </c>
+      <c r="P12" s="36">
+        <v>2.0714441490435082E-4</v>
+      </c>
+      <c r="Q12" s="36">
+        <v>0.18554040818080225</v>
+      </c>
+      <c r="R12" s="36">
+        <v>9.7916639130009184E-2</v>
+      </c>
+      <c r="S12" s="36">
+        <v>3.5981148291444105E-4</v>
+      </c>
+      <c r="T12" s="36">
+        <v>8.2140102854375322E-4</v>
+      </c>
+      <c r="U12" s="36">
+        <v>2.0656198979983266E-4</v>
+      </c>
+    </row>
+    <row r="13" spans="1:21" x14ac:dyDescent="0.35">
+      <c r="A13" s="36" t="s">
+        <v>39</v>
+      </c>
+      <c r="B13" s="36">
+        <v>12.52083577437433</v>
+      </c>
+      <c r="C13" s="36">
+        <v>20.270532842795603</v>
+      </c>
+      <c r="D13" s="36">
+        <v>0.3409180172553668</v>
+      </c>
+      <c r="E13" s="36">
+        <v>2.9109095355928769</v>
+      </c>
+      <c r="F13" s="36">
+        <v>0.2497973913339373</v>
+      </c>
+      <c r="G13" s="36">
+        <v>13.124249546633333</v>
+      </c>
+      <c r="H13" s="36">
+        <v>21.247425991845997</v>
+      </c>
+      <c r="I13" s="36">
+        <v>2.748829240149853E-2</v>
+      </c>
+      <c r="J13" s="36">
+        <v>1.2565609806706216E-2</v>
+      </c>
+      <c r="K13" s="36">
+        <v>2.2745794317306469E-2</v>
+      </c>
+      <c r="L13" s="36">
+        <v>12.52083577437433</v>
+      </c>
+      <c r="M13" s="36">
+        <v>20.270532842795603</v>
+      </c>
+      <c r="N13" s="36">
+        <v>2.6224462865797448E-2</v>
+      </c>
+      <c r="O13" s="36">
+        <v>2.2391611812252892E-2</v>
+      </c>
+      <c r="P13" s="36">
+        <v>2.1693922889409144E-2</v>
+      </c>
+      <c r="Q13" s="36">
+        <v>12.52083577437433</v>
+      </c>
+      <c r="R13" s="36">
+        <v>7.7224571792174466</v>
+      </c>
+      <c r="S13" s="36">
+        <v>2.6224462865797448E-2</v>
+      </c>
+      <c r="T13" s="36">
+        <v>2.2391611812252892E-2</v>
+      </c>
+      <c r="U13" s="36">
+        <v>2.0923767349099655E-2</v>
+      </c>
+    </row>
+    <row r="14" spans="1:21" x14ac:dyDescent="0.35">
+      <c r="A14" s="36" t="s">
+        <v>40</v>
+      </c>
+      <c r="B14" s="36">
+        <v>6.7241593267508967E-3</v>
+      </c>
+      <c r="C14" s="36">
+        <v>1.1779684094294906E-2</v>
+      </c>
+      <c r="D14" s="36">
+        <v>3.8796899778191691E-4</v>
+      </c>
+      <c r="E14" s="36">
+        <v>1.4617859597280451E-2</v>
+      </c>
+      <c r="F14" s="36">
+        <v>2.1012490503014364E-4</v>
+      </c>
+      <c r="G14" s="36">
+        <v>7.0482151979196148E-3</v>
+      </c>
+      <c r="H14" s="36">
+        <v>1.2347379713297071E-2</v>
+      </c>
+      <c r="I14" s="36">
+        <v>3.1282022990756972E-5</v>
+      </c>
+      <c r="J14" s="36">
+        <v>6.310134947949541E-5</v>
+      </c>
+      <c r="K14" s="36">
+        <v>1.8516047309667963E-5</v>
+      </c>
+      <c r="L14" s="36">
+        <v>6.7241593267508967E-3</v>
+      </c>
+      <c r="M14" s="36">
+        <v>1.1779684094294906E-2</v>
+      </c>
+      <c r="N14" s="36">
+        <v>2.984376906014746E-5</v>
+      </c>
+      <c r="O14" s="36">
+        <v>1.1244507382523421E-4</v>
+      </c>
+      <c r="P14" s="36">
+        <v>1.7664651554648802E-5</v>
+      </c>
+      <c r="Q14" s="36">
+        <v>6.7241593267508967E-3</v>
+      </c>
+      <c r="R14" s="36">
+        <v>5.8499541594588169E-3</v>
+      </c>
+      <c r="S14" s="36">
+        <v>2.984376906014746E-5</v>
+      </c>
+      <c r="T14" s="36">
+        <v>1.1244507382523421E-4</v>
+      </c>
+      <c r="U14" s="36">
+        <v>1.7144903019630951E-5</v>
+      </c>
+    </row>
+    <row r="15" spans="1:21" x14ac:dyDescent="0.35">
+      <c r="A15" s="36" t="s">
+        <v>41</v>
+      </c>
+      <c r="B15" s="36">
+        <v>1.1156981870757789E-2</v>
+      </c>
+      <c r="C15" s="36">
+        <v>2.9393646453474143E-3</v>
+      </c>
+      <c r="D15" s="36">
+        <v>1.5301644660926006E-4</v>
+      </c>
+      <c r="E15" s="36">
+        <v>4.9498784421843885E-3</v>
+      </c>
+      <c r="F15" s="36">
+        <v>1.0377034733426545E-4</v>
+      </c>
+      <c r="G15" s="36">
+        <v>1.1694667744047321E-2</v>
+      </c>
+      <c r="H15" s="36">
+        <v>3.0810207728340371E-3</v>
+      </c>
+      <c r="I15" s="36">
+        <v>1.2337748707141451E-5</v>
+      </c>
+      <c r="J15" s="36">
+        <v>2.1367287555519198E-5</v>
+      </c>
+      <c r="K15" s="36">
+        <v>9.2695275066846165E-6</v>
+      </c>
+      <c r="L15" s="36">
+        <v>1.1156981870757789E-2</v>
+      </c>
+      <c r="M15" s="36">
+        <v>2.9393646453474143E-3</v>
+      </c>
+      <c r="N15" s="36">
+        <v>1.1770495893020006E-5</v>
+      </c>
+      <c r="O15" s="36">
+        <v>3.8075988016802985E-5</v>
+      </c>
+      <c r="P15" s="36">
+        <v>8.8422522079635194E-6</v>
+      </c>
+      <c r="Q15" s="36">
+        <v>1.1156981870757789E-2</v>
+      </c>
+      <c r="R15" s="36">
+        <v>1.6046475309460435E-3</v>
+      </c>
+      <c r="S15" s="36">
+        <v>1.1770495893020006E-5</v>
+      </c>
+      <c r="T15" s="36">
+        <v>3.8075988016802985E-5</v>
+      </c>
+      <c r="U15" s="36">
+        <v>8.5601192917414183E-6</v>
+      </c>
+    </row>
+    <row r="16" spans="1:21" x14ac:dyDescent="0.35">
+      <c r="A16" s="36" t="s">
+        <v>42</v>
+      </c>
+      <c r="B16" s="36">
+        <v>0.49072032206537136</v>
+      </c>
+      <c r="C16" s="36">
+        <v>0.66823495038723257</v>
+      </c>
+      <c r="D16" s="36">
+        <v>1.5054465154747764E-2</v>
+      </c>
+      <c r="E16" s="36">
+        <v>10.387608134212732</v>
+      </c>
+      <c r="F16" s="36">
+        <v>2.3743380229952097E-2</v>
+      </c>
+      <c r="G16" s="36">
+        <v>0.51436949421310008</v>
+      </c>
+      <c r="H16" s="36">
+        <v>0.70043904438179805</v>
+      </c>
+      <c r="I16" s="36">
+        <v>1.2138447344421275E-3</v>
+      </c>
+      <c r="J16" s="36">
+        <v>4.4840497117303882E-2</v>
+      </c>
+      <c r="K16" s="36">
+        <v>2.03988188433999E-3</v>
+      </c>
+      <c r="L16" s="36">
+        <v>0.49072032206537136</v>
+      </c>
+      <c r="M16" s="36">
+        <v>0.66823495038723257</v>
+      </c>
+      <c r="N16" s="36">
+        <v>1.1580357811344436E-3</v>
+      </c>
+      <c r="O16" s="36">
+        <v>7.9904677955482534E-2</v>
+      </c>
+      <c r="P16" s="36">
+        <v>1.946020017423824E-3</v>
+      </c>
+      <c r="Q16" s="36">
+        <v>0.49072032206537136</v>
+      </c>
+      <c r="R16" s="36">
+        <v>0.13987738114791087</v>
+      </c>
+      <c r="S16" s="36">
+        <v>1.1580357811344436E-3</v>
+      </c>
+      <c r="T16" s="36">
+        <v>7.9904677955482534E-2</v>
+      </c>
+      <c r="U16" s="36">
+        <v>1.908764859368167E-3</v>
+      </c>
+    </row>
+    <row r="17" spans="1:21" x14ac:dyDescent="0.35">
+      <c r="A17" s="36" t="s">
+        <v>43</v>
+      </c>
+      <c r="B17" s="36">
+        <v>1.0122770216150535E-2</v>
+      </c>
+      <c r="C17" s="36">
+        <v>1.8688300667757635E-2</v>
+      </c>
+      <c r="D17" s="36">
+        <v>4.0166511852582403E-4</v>
+      </c>
+      <c r="E17" s="36">
+        <v>6.9341268212173074E-3</v>
+      </c>
+      <c r="F17" s="36">
+        <v>6.9243587856217465E-4</v>
+      </c>
+      <c r="G17" s="36">
+        <v>1.0610614563916826E-2</v>
+      </c>
+      <c r="H17" s="36">
+        <v>1.9588941663794147E-2</v>
+      </c>
+      <c r="I17" s="36">
+        <v>3.2386344125807871E-5</v>
+      </c>
+      <c r="J17" s="36">
+        <v>2.9932751574805081E-5</v>
+      </c>
+      <c r="K17" s="36">
+        <v>6.7405937097283868E-5</v>
+      </c>
+      <c r="L17" s="36">
+        <v>1.0122770216150535E-2</v>
+      </c>
+      <c r="M17" s="36">
+        <v>1.8688300667757635E-2</v>
+      </c>
+      <c r="N17" s="36">
+        <v>3.0897316809678778E-5</v>
+      </c>
+      <c r="O17" s="36">
+        <v>5.3339437086286976E-5</v>
+      </c>
+      <c r="P17" s="36">
+        <v>6.4281046842151228E-5</v>
+      </c>
+      <c r="Q17" s="36">
+        <v>1.0122770216150535E-2</v>
+      </c>
+      <c r="R17" s="36">
+        <v>5.931113933515357E-3</v>
+      </c>
+      <c r="S17" s="36">
+        <v>3.0897316809678778E-5</v>
+      </c>
+      <c r="T17" s="36">
+        <v>5.3339437086286976E-5</v>
+      </c>
+      <c r="U17" s="36">
+        <v>6.0668138442170768E-5</v>
+      </c>
+    </row>
+    <row r="18" spans="1:21" x14ac:dyDescent="0.35">
+      <c r="A18" s="36" t="s">
+        <v>44</v>
+      </c>
+      <c r="B18" s="36">
+        <v>4.4078201004555784E-2</v>
+      </c>
+      <c r="C18" s="36">
+        <v>4.1106878812466115E-2</v>
+      </c>
+      <c r="D18" s="36">
+        <v>1.0191057553681857E-3</v>
+      </c>
+      <c r="E18" s="36">
+        <v>1.5513132229614854E-2</v>
+      </c>
+      <c r="F18" s="36">
+        <v>1.734446323448037E-3</v>
+      </c>
+      <c r="G18" s="36">
+        <v>4.6202451655377751E-2</v>
+      </c>
+      <c r="H18" s="36">
+        <v>4.3087933213066892E-2</v>
+      </c>
+      <c r="I18" s="36">
+        <v>8.2170714288259651E-5</v>
+      </c>
+      <c r="J18" s="36">
+        <v>6.6965999490422535E-5</v>
+      </c>
+      <c r="K18" s="36">
+        <v>1.6098240812903258E-4</v>
+      </c>
+      <c r="L18" s="36">
+        <v>4.4078201004555784E-2</v>
+      </c>
+      <c r="M18" s="36">
+        <v>4.1106878812466115E-2</v>
+      </c>
+      <c r="N18" s="36">
+        <v>7.8392750412937374E-5</v>
+      </c>
+      <c r="O18" s="36">
+        <v>1.1933178638165271E-4</v>
+      </c>
+      <c r="P18" s="36">
+        <v>1.5354811679026028E-4</v>
+      </c>
+      <c r="Q18" s="36">
+        <v>4.4078201004555784E-2</v>
+      </c>
+      <c r="R18" s="36">
+        <v>4.4377525664870722E-2</v>
+      </c>
+      <c r="S18" s="36">
+        <v>7.8392750412937374E-5</v>
+      </c>
+      <c r="T18" s="36">
+        <v>1.1933178638165271E-4</v>
+      </c>
+      <c r="U18" s="36">
+        <v>1.468274983081093E-4</v>
+      </c>
+    </row>
+    <row r="19" spans="1:21" x14ac:dyDescent="0.35">
+      <c r="A19" s="36" t="s">
+        <v>45</v>
+      </c>
+      <c r="B19" s="36">
+        <v>3.5943868129653479E-2</v>
+      </c>
+      <c r="C19" s="36">
+        <v>4.1600737674390056E-2</v>
+      </c>
+      <c r="D19" s="36">
+        <v>0.21419720287398614</v>
+      </c>
+      <c r="E19" s="36">
+        <v>1.6813412403075465E-2</v>
+      </c>
+      <c r="F19" s="36">
+        <v>-0.19175909996212889</v>
+      </c>
+      <c r="G19" s="36">
+        <v>3.7676102738311477E-2</v>
+      </c>
+      <c r="H19" s="36">
+        <v>4.3605592502071508E-2</v>
+      </c>
+      <c r="I19" s="36">
+        <v>1.7270766126076732E-2</v>
+      </c>
+      <c r="J19" s="36">
+        <v>7.2578957605170163E-5</v>
+      </c>
+      <c r="K19" s="36">
+        <v>-1.6247417482315733E-2</v>
+      </c>
+      <c r="L19" s="36">
+        <v>3.5943868129653479E-2</v>
+      </c>
+      <c r="M19" s="36">
+        <v>4.1600737674390056E-2</v>
+      </c>
+      <c r="N19" s="36">
+        <v>1.647670791338355E-2</v>
+      </c>
+      <c r="O19" s="36">
+        <v>1.2933394156211894E-4</v>
+      </c>
+      <c r="P19" s="36">
+        <v>-1.5562079225600212E-2</v>
+      </c>
+      <c r="Q19" s="36">
+        <v>3.5943868129653479E-2</v>
+      </c>
+      <c r="R19" s="36">
+        <v>2.9518986200011123E-2</v>
+      </c>
+      <c r="S19" s="36">
+        <v>1.647670791338355E-2</v>
+      </c>
+      <c r="T19" s="36">
+        <v>1.2933394156211894E-4</v>
+      </c>
+      <c r="U19" s="36">
+        <v>-1.4879393989363563E-2</v>
+      </c>
+    </row>
+    <row r="20" spans="1:21" x14ac:dyDescent="0.35">
+      <c r="A20" s="36" t="s">
+        <v>46</v>
+      </c>
+      <c r="B20" s="36">
+        <v>28.740220857776386</v>
+      </c>
+      <c r="C20" s="36">
+        <v>33.798432508318513</v>
+      </c>
+      <c r="D20" s="36">
+        <v>0.85667244994842429</v>
+      </c>
+      <c r="E20" s="36">
+        <v>476.6582849154841</v>
+      </c>
+      <c r="F20" s="36">
+        <v>0</v>
+      </c>
+      <c r="G20" s="36">
+        <v>30.125291742488503</v>
+      </c>
+      <c r="H20" s="36">
+        <v>35.427272629201333</v>
+      </c>
+      <c r="I20" s="36">
+        <v>6.9073682247926718E-2</v>
+      </c>
+      <c r="J20" s="36">
+        <v>2.0576050015109337</v>
+      </c>
+      <c r="K20" s="36">
+        <v>0</v>
+      </c>
+      <c r="L20" s="36">
+        <v>28.740220857776386</v>
+      </c>
+      <c r="M20" s="36">
+        <v>33.798432508318513</v>
+      </c>
+      <c r="N20" s="36">
+        <v>6.5897880765263414E-2</v>
+      </c>
+      <c r="O20" s="36">
+        <v>3.6666021916575695</v>
+      </c>
+      <c r="P20" s="36">
+        <v>0</v>
+      </c>
+      <c r="Q20" s="36">
+        <v>28.740220857776386</v>
+      </c>
+      <c r="R20" s="36">
+        <v>8.4880818314284046</v>
+      </c>
+      <c r="S20" s="36">
+        <v>6.5897880765263414E-2</v>
+      </c>
+      <c r="T20" s="36">
+        <v>3.6666021916575695</v>
+      </c>
+      <c r="U20" s="36">
+        <v>0</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{997C2057-C145-4E74-9B2E-03F75EB3C059}">
+  <dimension ref="A1:M10"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetData>
+    <row r="1" spans="1:13" x14ac:dyDescent="0.35">
+      <c r="A1" s="58" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="59" t="s">
+        <v>47</v>
+      </c>
+      <c r="C1" s="60" t="s">
+        <v>47</v>
+      </c>
+      <c r="D1" s="60" t="s">
+        <v>47</v>
+      </c>
+      <c r="E1" s="60" t="s">
+        <v>47</v>
+      </c>
+      <c r="F1" s="61" t="s">
+        <v>47</v>
+      </c>
+      <c r="G1" s="59" t="s">
+        <v>48</v>
+      </c>
+      <c r="H1" s="59" t="s">
+        <v>48</v>
+      </c>
+      <c r="I1" s="59" t="s">
+        <v>48</v>
+      </c>
+      <c r="J1" s="59" t="s">
+        <v>48</v>
+      </c>
+      <c r="K1" s="59" t="s">
+        <v>49</v>
+      </c>
+      <c r="L1" s="59" t="s">
+        <v>49</v>
+      </c>
+      <c r="M1" s="59" t="s">
+        <v>49</v>
+      </c>
+    </row>
+    <row r="2" spans="1:13" x14ac:dyDescent="0.35">
+      <c r="A2" s="62"/>
+      <c r="B2" s="63" t="s">
+        <v>50</v>
+      </c>
+      <c r="C2" s="64" t="s">
+        <v>51</v>
+      </c>
+      <c r="D2" s="64" t="s">
+        <v>52</v>
+      </c>
+      <c r="E2" s="64" t="s">
+        <v>53</v>
+      </c>
+      <c r="F2" s="65" t="s">
+        <v>54</v>
+      </c>
+      <c r="G2" s="63" t="s">
+        <v>50</v>
+      </c>
+      <c r="H2" s="64" t="s">
+        <v>55</v>
+      </c>
+      <c r="I2" s="64" t="s">
+        <v>56</v>
+      </c>
+      <c r="J2" s="65" t="s">
+        <v>57</v>
+      </c>
+      <c r="K2" s="63" t="s">
+        <v>51</v>
+      </c>
+      <c r="L2" s="64" t="s">
+        <v>58</v>
+      </c>
+      <c r="M2" s="65" t="s">
+        <v>59</v>
+      </c>
+    </row>
+    <row r="3" spans="1:13" x14ac:dyDescent="0.35">
+      <c r="A3" s="58" t="s">
+        <v>60</v>
+      </c>
+      <c r="B3" s="66">
+        <v>0.2</v>
+      </c>
+      <c r="C3" s="67">
+        <v>5.2</v>
+      </c>
+      <c r="D3" s="67">
+        <v>3.2</v>
+      </c>
+      <c r="E3" s="67">
+        <v>1</v>
+      </c>
+      <c r="F3" s="68">
+        <v>2E-3</v>
+      </c>
+      <c r="G3" s="66">
+        <v>2.77</v>
+      </c>
+      <c r="H3" s="67">
+        <v>2.1</v>
+      </c>
+      <c r="I3" s="67">
+        <v>0</v>
+      </c>
+      <c r="J3" s="68">
+        <v>0.02</v>
+      </c>
+      <c r="K3" s="66">
+        <v>6.7</v>
+      </c>
+      <c r="L3" s="67">
+        <v>0.45</v>
+      </c>
+      <c r="M3" s="68">
+        <v>0.5</v>
+      </c>
+    </row>
+    <row r="4" spans="1:13" x14ac:dyDescent="0.35">
+      <c r="A4" s="58" t="s">
+        <v>61</v>
+      </c>
+      <c r="B4" s="69">
+        <v>9.62332812</v>
+      </c>
+      <c r="C4" s="70">
+        <v>18.183705960000001</v>
+      </c>
+      <c r="D4" s="70">
+        <v>9.8108925599999992</v>
+      </c>
+      <c r="E4" s="70">
+        <v>14.36153292</v>
+      </c>
+      <c r="F4" s="71">
+        <v>29.474569319999997</v>
+      </c>
+      <c r="G4" s="69">
+        <v>1.46512212</v>
+      </c>
+      <c r="H4" s="70">
+        <v>12.216521520000001</v>
+      </c>
+      <c r="I4" s="70">
+        <v>9.85031392970102</v>
+      </c>
+      <c r="J4" s="71">
+        <v>0.68795003364644203</v>
+      </c>
+      <c r="K4" s="69">
+        <v>1.70723384624563</v>
+      </c>
+      <c r="L4" s="70">
+        <v>0.44773587697512185</v>
+      </c>
+      <c r="M4" s="71">
+        <v>0.39331615887716798</v>
+      </c>
+    </row>
+    <row r="5" spans="1:13" x14ac:dyDescent="0.35">
+      <c r="A5" s="58" t="s">
+        <v>62</v>
+      </c>
+      <c r="B5" s="69">
+        <v>2.4228120000000002E-2</v>
+      </c>
+      <c r="C5" s="70">
+        <v>4.8495719999999999E-2</v>
+      </c>
+      <c r="D5" s="70">
+        <v>1.6290119999999998E-2</v>
+      </c>
+      <c r="E5" s="70">
+        <v>6.777119999999999E-2</v>
+      </c>
+      <c r="F5" s="71">
+        <v>0.11712455999999999</v>
+      </c>
+      <c r="G5" s="69">
+        <v>1.47E-4</v>
+      </c>
+      <c r="H5" s="70">
+        <v>0</v>
+      </c>
+      <c r="I5" s="70">
+        <v>2.47999284436436E-2</v>
+      </c>
+      <c r="J5" s="71">
+        <v>1.60093815024771E-3</v>
+      </c>
+      <c r="K5" s="69">
+        <v>2.7952697501062401E-3</v>
+      </c>
+      <c r="L5" s="70">
+        <v>1.4580968683355281E-3</v>
+      </c>
+      <c r="M5" s="71">
+        <v>1.3328185258781799E-3</v>
+      </c>
+    </row>
+    <row r="6" spans="1:13" x14ac:dyDescent="0.35">
+      <c r="A6" s="58" t="s">
+        <v>63</v>
+      </c>
+      <c r="B6" s="69">
+        <v>1.54477848</v>
+      </c>
+      <c r="C6" s="70">
+        <v>0.71068031999999992</v>
+      </c>
+      <c r="D6" s="70">
+        <v>0.48488495999999998</v>
+      </c>
+      <c r="E6" s="70">
+        <v>1.3786038</v>
+      </c>
+      <c r="F6" s="71">
+        <v>9.4698408000000001</v>
+      </c>
+      <c r="G6" s="69">
+        <v>4.2588000000000001E-3</v>
+      </c>
+      <c r="H6" s="70">
+        <v>0</v>
+      </c>
+      <c r="I6" s="70">
+        <v>1.5812148810503099</v>
+      </c>
+      <c r="J6" s="71">
+        <v>0.11209099583156799</v>
+      </c>
+      <c r="K6" s="69">
+        <v>0.257622178441546</v>
+      </c>
+      <c r="L6" s="70">
+        <v>5.9912377166165286E-2</v>
+      </c>
+      <c r="M6" s="71">
+        <v>1.5538321572476801</v>
+      </c>
+    </row>
+    <row r="7" spans="1:13" x14ac:dyDescent="0.35">
+      <c r="A7" s="58" t="s">
+        <v>64</v>
+      </c>
+      <c r="B7" s="69">
+        <v>2.52E-6</v>
+      </c>
+      <c r="C7" s="70">
+        <v>1.68E-6</v>
+      </c>
+      <c r="D7" s="70">
+        <v>1.68E-6</v>
+      </c>
+      <c r="E7" s="70">
+        <v>1.5119999999999999E-5</v>
+      </c>
+      <c r="F7" s="71">
+        <v>1.5119999999999999E-5</v>
+      </c>
+      <c r="G7" s="69">
+        <v>0</v>
+      </c>
+      <c r="H7" s="70">
+        <v>0</v>
+      </c>
+      <c r="I7" s="70">
+        <v>2.5135737237962902E-6</v>
+      </c>
+      <c r="J7" s="71">
+        <v>1.18416748899613E-7</v>
+      </c>
+      <c r="K7" s="69">
+        <v>2.5872237119058998E-7</v>
+      </c>
+      <c r="L7" s="70">
+        <v>2.033754680622914E-7</v>
+      </c>
+      <c r="M7" s="71">
+        <v>1.06984724644635E-7</v>
+      </c>
+    </row>
+    <row r="8" spans="1:13" x14ac:dyDescent="0.35">
+      <c r="A8" s="58" t="s">
+        <v>65</v>
+      </c>
+      <c r="B8" s="69">
+        <v>1.1664240000000001E-2</v>
+      </c>
+      <c r="C8" s="70">
+        <v>2.0127240000000001E-2</v>
+      </c>
+      <c r="D8" s="70">
+        <v>6.3176399999999994E-3</v>
+      </c>
+      <c r="E8" s="70">
+        <v>2.5383120000000002E-2</v>
+      </c>
+      <c r="F8" s="71">
+        <v>6.668592000000001E-2</v>
+      </c>
+      <c r="G8" s="69">
+        <v>5.4599999999999999E-5</v>
+      </c>
+      <c r="H8" s="70">
+        <v>0</v>
+      </c>
+      <c r="I8" s="70">
+        <v>1.19391674029994E-2</v>
+      </c>
+      <c r="J8" s="71">
+        <v>6.7644162062873001E-4</v>
+      </c>
+      <c r="K8" s="69">
+        <v>1.10330541338673E-3</v>
+      </c>
+      <c r="L8" s="70">
+        <v>6.030057782641262E-4</v>
+      </c>
+      <c r="M8" s="71">
+        <v>1.0333089972417301E-3</v>
+      </c>
+    </row>
+    <row r="9" spans="1:13" x14ac:dyDescent="0.35">
+      <c r="A9" s="58" t="s">
+        <v>66</v>
+      </c>
+      <c r="B9" s="69">
+        <v>8.9100479999999996E-2</v>
+      </c>
+      <c r="C9" s="70">
+        <v>0.24190068000000003</v>
+      </c>
+      <c r="D9" s="70">
+        <v>5.4098519999999997E-2</v>
+      </c>
+      <c r="E9" s="70">
+        <v>0.54149508000000002</v>
+      </c>
+      <c r="F9" s="71">
+        <v>0.67089288000000002</v>
+      </c>
+      <c r="G9" s="69">
+        <v>9.9372000000000002E-4</v>
+      </c>
+      <c r="H9" s="70">
+        <v>0</v>
+      </c>
+      <c r="I9" s="70">
+        <v>9.1201986373668095E-2</v>
+      </c>
+      <c r="J9" s="71">
+        <v>2.82054816290286E-3</v>
+      </c>
+      <c r="K9" s="69">
+        <v>9.6823553171410896E-3</v>
+      </c>
+      <c r="L9" s="70">
+        <v>6.0571574682519213E-3</v>
+      </c>
+      <c r="M9" s="71">
+        <v>3.0275083841827801E-3</v>
+      </c>
+    </row>
+    <row r="10" spans="1:13" ht="15" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="A10" s="58" t="s">
+        <v>67</v>
+      </c>
+      <c r="B10" s="72">
+        <v>3.4684255199999998</v>
+      </c>
+      <c r="C10" s="73">
+        <v>10.675000559999999</v>
+      </c>
+      <c r="D10" s="73">
+        <v>1.6516634399999999</v>
+      </c>
+      <c r="E10" s="73">
+        <v>4.32636792</v>
+      </c>
+      <c r="F10" s="74">
+        <v>7.9673496000000004</v>
+      </c>
+      <c r="G10" s="72">
+        <v>6.9896400000000001E-3</v>
+      </c>
+      <c r="H10" s="73">
+        <v>0</v>
+      </c>
+      <c r="I10" s="73">
+        <v>3.5502351524805098</v>
+      </c>
+      <c r="J10" s="74">
+        <v>0.34990442358520801</v>
+      </c>
+      <c r="K10" s="72">
+        <v>0.29111421187407199</v>
+      </c>
+      <c r="L10" s="73">
+        <v>0.1245111955582438</v>
+      </c>
+      <c r="M10" s="74">
+        <v>9.3423865648273097E-2</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{BB1DF6C3-C927-4831-B286-2F43E817A000}">
+  <dimension ref="A1:K19"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetData>
+    <row r="1" spans="1:11" ht="73" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="A1" s="75"/>
+      <c r="B1" s="76" t="s">
+        <v>68</v>
+      </c>
+      <c r="C1" s="76" t="s">
+        <v>68</v>
+      </c>
+      <c r="D1" s="76" t="s">
+        <v>68</v>
+      </c>
+      <c r="E1" s="76" t="s">
+        <v>68</v>
+      </c>
+      <c r="F1" s="76" t="s">
+        <v>68</v>
+      </c>
+      <c r="G1" s="76" t="s">
+        <v>69</v>
+      </c>
+      <c r="H1" s="76" t="s">
+        <v>69</v>
+      </c>
+      <c r="I1" s="76" t="s">
+        <v>69</v>
+      </c>
+      <c r="J1" s="76" t="s">
+        <v>69</v>
+      </c>
+      <c r="K1" s="76" t="s">
+        <v>69</v>
+      </c>
+    </row>
+    <row r="2" spans="1:11" ht="44" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="A2" s="77"/>
+      <c r="B2" s="78" t="s">
+        <v>23</v>
+      </c>
+      <c r="C2" s="78" t="s">
+        <v>24</v>
+      </c>
+      <c r="D2" s="78" t="s">
+        <v>25</v>
+      </c>
+      <c r="E2" s="78" t="s">
+        <v>26</v>
+      </c>
+      <c r="F2" s="78" t="s">
+        <v>27</v>
+      </c>
+      <c r="G2" s="78" t="s">
+        <v>23</v>
+      </c>
+      <c r="H2" s="78" t="s">
+        <v>24</v>
+      </c>
+      <c r="I2" s="78" t="s">
+        <v>25</v>
+      </c>
+      <c r="J2" s="78" t="s">
+        <v>26</v>
+      </c>
+      <c r="K2" s="78" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="3" spans="1:11" ht="15" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="A3" s="79" t="s">
+        <v>70</v>
+      </c>
+      <c r="B3" s="80">
+        <v>1.7709494059999999</v>
+      </c>
+      <c r="C3" s="80">
+        <v>2.6686453769999998</v>
+      </c>
+      <c r="D3" s="80">
+        <v>5.7663952999999997E-2</v>
+      </c>
+      <c r="E3" s="80">
+        <v>25.412554750000002</v>
+      </c>
+      <c r="F3" s="80">
+        <v>0.79790850400000002</v>
+      </c>
+      <c r="G3" s="80">
+        <v>1.856296366</v>
+      </c>
+      <c r="H3" s="80">
+        <v>2.797254793</v>
+      </c>
+      <c r="I3" s="80">
+        <v>4.6494570000000001E-3</v>
+      </c>
+      <c r="J3" s="80">
+        <v>0.10969913100000001</v>
+      </c>
+      <c r="K3" s="80">
+        <v>0.77155671599999998</v>
+      </c>
+    </row>
+    <row r="4" spans="1:11" ht="15" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="A4" s="79" t="s">
+        <v>71</v>
+      </c>
+      <c r="B4" s="80">
+        <v>1.46537E-6</v>
+      </c>
+      <c r="C4" s="80">
+        <v>9.9801499999999996E-6</v>
+      </c>
+      <c r="D4" s="80">
+        <v>5.6335799999999998E-8</v>
+      </c>
+      <c r="E4" s="80">
+        <v>7.1310799999999997E-6</v>
+      </c>
+      <c r="F4" s="80">
+        <v>2.68986E-5</v>
+      </c>
+      <c r="G4" s="80">
+        <v>1.5359899999999999E-6</v>
+      </c>
+      <c r="H4" s="80">
+        <v>1.0461100000000001E-5</v>
+      </c>
+      <c r="I4" s="80">
+        <v>4.5423699999999999E-9</v>
+      </c>
+      <c r="J4" s="80">
+        <v>3.07829E-8</v>
+      </c>
+      <c r="K4" s="80">
+        <v>2.82552E-5</v>
+      </c>
+    </row>
+    <row r="5" spans="1:11" ht="15" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="A5" s="79" t="s">
+        <v>72</v>
+      </c>
+      <c r="B5" s="80">
+        <v>4.3737649999999999E-3</v>
+      </c>
+      <c r="C5" s="80">
+        <v>3.6151059999999999E-3</v>
+      </c>
+      <c r="D5" s="80">
+        <v>1.19763E-4</v>
+      </c>
+      <c r="E5" s="80">
+        <v>1.866104E-2</v>
+      </c>
+      <c r="F5" s="80">
+        <v>2.00507E-4</v>
+      </c>
+      <c r="G5" s="80">
+        <v>4.5845490000000003E-3</v>
+      </c>
+      <c r="H5" s="80">
+        <v>3.7893279999999998E-3</v>
+      </c>
+      <c r="I5" s="80">
+        <v>9.6565399999999992E-6</v>
+      </c>
+      <c r="J5" s="80">
+        <v>8.0554699999999996E-5</v>
+      </c>
+      <c r="K5" s="80">
+        <v>1.75503E-5</v>
+      </c>
+    </row>
+    <row r="6" spans="1:11" ht="15" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="A6" s="79" t="s">
+        <v>73</v>
+      </c>
+      <c r="B6" s="80">
+        <v>4.4335889999999999E-3</v>
+      </c>
+      <c r="C6" s="80">
+        <v>3.7010300000000001E-3</v>
+      </c>
+      <c r="D6" s="80">
+        <v>1.2176399999999999E-4</v>
+      </c>
+      <c r="E6" s="80">
+        <v>1.9364396999999998E-2</v>
+      </c>
+      <c r="F6" s="80">
+        <v>2.08736E-4</v>
+      </c>
+      <c r="G6" s="80">
+        <v>4.6472559999999998E-3</v>
+      </c>
+      <c r="H6" s="80">
+        <v>3.8793930000000001E-3</v>
+      </c>
+      <c r="I6" s="80">
+        <v>9.8178900000000006E-6</v>
+      </c>
+      <c r="J6" s="80">
+        <v>8.35909E-5</v>
+      </c>
+      <c r="K6" s="80">
+        <v>1.8258400000000001E-5</v>
+      </c>
+    </row>
+    <row r="7" spans="1:11" ht="15" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="A7" s="79" t="s">
+        <v>74</v>
+      </c>
+      <c r="B7" s="80">
+        <v>0.19976666000000001</v>
+      </c>
+      <c r="C7" s="80">
+        <v>9.1455141000000004E-2</v>
+      </c>
+      <c r="D7" s="80">
+        <v>5.3663069999999998E-3</v>
+      </c>
+      <c r="E7" s="80">
+        <v>0.111130149</v>
+      </c>
+      <c r="F7" s="80">
+        <v>1.1594619E-2</v>
+      </c>
+      <c r="G7" s="80">
+        <v>0.20939396900000001</v>
+      </c>
+      <c r="H7" s="80">
+        <v>9.5862616999999997E-2</v>
+      </c>
+      <c r="I7" s="80">
+        <v>4.32686E-4</v>
+      </c>
+      <c r="J7" s="80">
+        <v>4.7971899999999998E-4</v>
+      </c>
+      <c r="K7" s="80">
+        <v>9.7354400000000002E-4</v>
+      </c>
+    </row>
+    <row r="8" spans="1:11" ht="15" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="A8" s="79" t="s">
+        <v>75</v>
+      </c>
+      <c r="B8" s="80">
+        <v>0.148875913</v>
+      </c>
+      <c r="C8" s="80">
+        <v>0.19170925</v>
+      </c>
+      <c r="D8" s="80">
+        <v>6.8379720000000003E-3</v>
+      </c>
+      <c r="E8" s="80">
+        <v>0.170138662</v>
+      </c>
+      <c r="F8" s="80">
+        <v>5.5954430000000003E-3</v>
+      </c>
+      <c r="G8" s="80">
+        <v>0.15605065600000001</v>
+      </c>
+      <c r="H8" s="80">
+        <v>0.20094824999999999</v>
+      </c>
+      <c r="I8" s="80">
+        <v>5.5134699999999999E-4</v>
+      </c>
+      <c r="J8" s="80">
+        <v>7.3444299999999999E-4</v>
+      </c>
+      <c r="K8" s="80">
+        <v>4.7602300000000001E-4</v>
+      </c>
+    </row>
+    <row r="9" spans="1:11" x14ac:dyDescent="0.35">
+      <c r="A9" s="81" t="s">
+        <v>76</v>
+      </c>
+      <c r="B9" s="82">
+        <v>2.7490001309999998</v>
+      </c>
+      <c r="C9" s="82">
+        <v>3.5593597469999998</v>
+      </c>
+      <c r="D9" s="82">
+        <v>7.7236404999999994E-2</v>
+      </c>
+      <c r="E9" s="82">
+        <v>0.80830365100000001</v>
+      </c>
+      <c r="F9" s="82">
+        <v>5.0465699000000003E-2</v>
+      </c>
+      <c r="G9" s="82">
+        <v>2.8814820650000001</v>
+      </c>
+      <c r="H9" s="82">
+        <v>3.7308951559999999</v>
+      </c>
+      <c r="I9" s="82">
+        <v>6.227588E-3</v>
+      </c>
+      <c r="J9" s="82">
+        <v>3.489228E-3</v>
+      </c>
+      <c r="K9" s="82">
+        <v>4.1773510000000002E-3</v>
+      </c>
+    </row>
+    <row r="10" spans="1:11" x14ac:dyDescent="0.35">
+      <c r="A10" s="83" t="s">
+        <v>77</v>
+      </c>
+      <c r="B10" s="84">
+        <v>0.14084532699999999</v>
+      </c>
+      <c r="C10" s="84">
+        <v>0.22035233600000001</v>
+      </c>
+      <c r="D10" s="84">
+        <v>3.4970869999999999E-3</v>
+      </c>
+      <c r="E10" s="84">
+        <v>4.7008515000000001E-2</v>
+      </c>
+      <c r="F10" s="84">
+        <v>1.837396E-3</v>
+      </c>
+      <c r="G10" s="84">
+        <v>0.14763305400000001</v>
+      </c>
+      <c r="H10" s="84">
+        <v>0.23097172599999999</v>
+      </c>
+      <c r="I10" s="84">
+        <v>2.81971E-4</v>
+      </c>
+      <c r="J10" s="84">
+        <v>2.0292300000000001E-4</v>
+      </c>
+      <c r="K10" s="84">
+        <v>1.50412E-4</v>
+      </c>
+    </row>
+    <row r="11" spans="1:11" x14ac:dyDescent="0.35">
+      <c r="A11" s="83" t="s">
+        <v>78</v>
+      </c>
+      <c r="B11" s="84">
+        <v>0.18554040799999999</v>
+      </c>
+      <c r="C11" s="84">
+        <v>0.28794463100000001</v>
+      </c>
+      <c r="D11" s="84">
+        <v>4.6775489999999996E-3</v>
+      </c>
+      <c r="E11" s="84">
+        <v>0.106782134</v>
+      </c>
+      <c r="F11" s="84">
+        <v>2.6382990000000002E-3</v>
+      </c>
+      <c r="G11" s="84">
+        <v>0.19448211500000001</v>
+      </c>
+      <c r="H11" s="84">
+        <v>0.301821481</v>
+      </c>
+      <c r="I11" s="84">
+        <v>3.7715200000000001E-4</v>
+      </c>
+      <c r="J11" s="84">
+        <v>4.6095000000000001E-4</v>
+      </c>
+      <c r="K11" s="84">
+        <v>2.1713099999999999E-4</v>
+      </c>
+    </row>
+    <row r="12" spans="1:11" x14ac:dyDescent="0.35">
+      <c r="A12" s="83" t="s">
+        <v>79</v>
+      </c>
+      <c r="B12" s="84">
+        <v>12.52083577</v>
+      </c>
+      <c r="C12" s="84">
+        <v>20.270532840000001</v>
+      </c>
+      <c r="D12" s="84">
+        <v>0.34091801700000002</v>
+      </c>
+      <c r="E12" s="84">
+        <v>2.9109095360000001</v>
+      </c>
+      <c r="F12" s="84">
+        <v>0.24979739100000001</v>
+      </c>
+      <c r="G12" s="84">
+        <v>13.12424955</v>
+      </c>
+      <c r="H12" s="84">
+        <v>21.24742599</v>
+      </c>
+      <c r="I12" s="84">
+        <v>2.7488292000000001E-2</v>
+      </c>
+      <c r="J12" s="84">
+        <v>1.256561E-2</v>
+      </c>
+      <c r="K12" s="84">
+        <v>2.2745794E-2</v>
+      </c>
+    </row>
+    <row r="13" spans="1:11" x14ac:dyDescent="0.35">
+      <c r="A13" s="83" t="s">
+        <v>80</v>
+      </c>
+      <c r="B13" s="84">
+        <v>6.7241590000000004E-3</v>
+      </c>
+      <c r="C13" s="84">
+        <v>1.1779684E-2</v>
+      </c>
+      <c r="D13" s="84">
+        <v>3.87969E-4</v>
+      </c>
+      <c r="E13" s="84">
+        <v>1.461786E-2</v>
+      </c>
+      <c r="F13" s="84">
+        <v>2.10125E-4</v>
+      </c>
+      <c r="G13" s="84">
+        <v>7.048215E-3</v>
+      </c>
+      <c r="H13" s="84">
+        <v>1.234738E-2</v>
+      </c>
+      <c r="I13" s="84">
+        <v>3.1282000000000003E-5</v>
+      </c>
+      <c r="J13" s="84">
+        <v>6.3101299999999998E-5</v>
+      </c>
+      <c r="K13" s="84">
+        <v>1.8516E-5</v>
+      </c>
+    </row>
+    <row r="14" spans="1:11" x14ac:dyDescent="0.35">
+      <c r="A14" s="83" t="s">
+        <v>81</v>
+      </c>
+      <c r="B14" s="84">
+        <v>1.1156981999999999E-2</v>
+      </c>
+      <c r="C14" s="84">
+        <v>2.9393650000000002E-3</v>
+      </c>
+      <c r="D14" s="84">
+        <v>1.5301600000000001E-4</v>
+      </c>
+      <c r="E14" s="84">
+        <v>4.9498779999999996E-3</v>
+      </c>
+      <c r="F14" s="84">
+        <v>1.0377E-4</v>
+      </c>
+      <c r="G14" s="84">
+        <v>1.1694668E-2</v>
+      </c>
+      <c r="H14" s="84">
+        <v>3.0810210000000002E-3</v>
+      </c>
+      <c r="I14" s="84">
+        <v>1.23377E-5</v>
+      </c>
+      <c r="J14" s="84">
+        <v>2.1367300000000001E-5</v>
+      </c>
+      <c r="K14" s="84">
+        <v>9.2695300000000003E-6</v>
+      </c>
+    </row>
+    <row r="15" spans="1:11" x14ac:dyDescent="0.35">
+      <c r="A15" s="83" t="s">
+        <v>82</v>
+      </c>
+      <c r="B15" s="84">
+        <v>0.49072032199999999</v>
+      </c>
+      <c r="C15" s="84">
+        <v>0.66823494999999999</v>
+      </c>
+      <c r="D15" s="84">
+        <v>1.5054465E-2</v>
+      </c>
+      <c r="E15" s="84">
+        <v>10.38760813</v>
+      </c>
+      <c r="F15" s="84">
+        <v>2.3743380000000001E-2</v>
+      </c>
+      <c r="G15" s="84">
+        <v>0.51436949399999998</v>
+      </c>
+      <c r="H15" s="84">
+        <v>0.70043904400000001</v>
+      </c>
+      <c r="I15" s="84">
+        <v>1.2138450000000001E-3</v>
+      </c>
+      <c r="J15" s="84">
+        <v>4.4840497E-2</v>
+      </c>
+      <c r="K15" s="84">
+        <v>2.0398819999999998E-3</v>
+      </c>
+    </row>
+    <row r="16" spans="1:11" x14ac:dyDescent="0.35">
+      <c r="A16" s="83" t="s">
+        <v>83</v>
+      </c>
+      <c r="B16" s="84">
+        <v>1.012277E-2</v>
+      </c>
+      <c r="C16" s="84">
+        <v>1.8688301000000001E-2</v>
+      </c>
+      <c r="D16" s="84">
+        <v>4.01665E-4</v>
+      </c>
+      <c r="E16" s="84">
+        <v>6.934127E-3</v>
+      </c>
+      <c r="F16" s="84">
+        <v>6.9243600000000005E-4</v>
+      </c>
+      <c r="G16" s="84">
+        <v>1.0610615E-2</v>
+      </c>
+      <c r="H16" s="84">
+        <v>1.9588942000000002E-2</v>
+      </c>
+      <c r="I16" s="84">
+        <v>3.2386299999999999E-5</v>
+      </c>
+      <c r="J16" s="84">
+        <v>2.9932799999999999E-5</v>
+      </c>
+      <c r="K16" s="84">
+        <v>6.7405900000000005E-5</v>
+      </c>
+    </row>
+    <row r="17" spans="1:11" x14ac:dyDescent="0.35">
+      <c r="A17" s="83" t="s">
+        <v>84</v>
+      </c>
+      <c r="B17" s="84">
+        <v>4.4078200999999997E-2</v>
+      </c>
+      <c r="C17" s="84">
+        <v>4.1106878999999999E-2</v>
+      </c>
+      <c r="D17" s="84">
+        <v>1.0191060000000001E-3</v>
+      </c>
+      <c r="E17" s="84">
+        <v>1.5513132000000001E-2</v>
+      </c>
+      <c r="F17" s="84">
+        <v>1.7344459999999999E-3</v>
+      </c>
+      <c r="G17" s="84">
+        <v>4.6202451999999998E-2</v>
+      </c>
+      <c r="H17" s="84">
+        <v>4.3087933000000002E-2</v>
+      </c>
+      <c r="I17" s="84">
+        <v>8.2170700000000003E-5</v>
+      </c>
+      <c r="J17" s="84">
+        <v>6.6965999999999995E-5</v>
+      </c>
+      <c r="K17" s="84">
+        <v>1.60982E-4</v>
+      </c>
+    </row>
+    <row r="18" spans="1:11" x14ac:dyDescent="0.35">
+      <c r="A18" s="83" t="s">
+        <v>85</v>
+      </c>
+      <c r="B18" s="84">
+        <v>3.5943867999999997E-2</v>
+      </c>
+      <c r="C18" s="84">
+        <v>4.1600737999999998E-2</v>
+      </c>
+      <c r="D18" s="84">
+        <v>0.13496461900000001</v>
+      </c>
+      <c r="E18" s="84">
+        <v>1.6813412E-2</v>
+      </c>
+      <c r="F18" s="84">
+        <v>-0.19175909999999999</v>
+      </c>
+      <c r="G18" s="84">
+        <v>3.7676103000000002E-2</v>
+      </c>
+      <c r="H18" s="84">
+        <v>4.3605592999999998E-2</v>
+      </c>
+      <c r="I18" s="84">
+        <v>1.0882226E-2</v>
+      </c>
+      <c r="J18" s="84">
+        <v>7.2578999999999997E-5</v>
+      </c>
+      <c r="K18" s="84">
+        <v>-1.6247417E-2</v>
+      </c>
+    </row>
+    <row r="19" spans="1:11" x14ac:dyDescent="0.35">
+      <c r="A19" s="83" t="s">
+        <v>86</v>
+      </c>
+      <c r="B19" s="84">
+        <v>28.740220860000001</v>
+      </c>
+      <c r="C19" s="84">
+        <v>33.798432509999998</v>
+      </c>
+      <c r="D19" s="84">
+        <v>0.85667245000000003</v>
+      </c>
+      <c r="E19" s="84">
+        <v>476.65828490000001</v>
+      </c>
+      <c r="F19" s="84">
+        <v>0</v>
+      </c>
+      <c r="G19" s="84">
+        <v>30.125291740000002</v>
+      </c>
+      <c r="H19" s="84">
+        <v>35.427272629999997</v>
+      </c>
+      <c r="I19" s="84">
+        <v>6.9073681999999997E-2</v>
+      </c>
+      <c r="J19" s="84">
+        <v>2.0576050019999998</v>
+      </c>
+      <c r="K19" s="84">
+        <v>0</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
 </file>
</xml_diff>